<commit_message>
Clarify annual returns in wide workbook
</commit_message>
<xml_diff>
--- a/analysis/forward_beat_curves_wide.xlsx
+++ b/analysis/forward_beat_curves_wide.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Beats Wide" sheetId="1" r:id="Raf67439f6fca4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Beats Wide" sheetId="1" r:id="R8699e01df06f4bda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -92,7 +92,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>All Long Beat</c:v>
+            <c:v>All Long Annual Return</c:v>
           </c:tx>
           <c:dLbls>
             <c:showLegendKey val="0"/>
@@ -126,7 +126,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>All Short Beat</c:v>
+            <c:v>All Long Beat</c:v>
           </c:tx>
           <c:dLbls>
             <c:showLegendKey val="0"/>
@@ -160,7 +160,7 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:v>Winner Long Beat</c:v>
+            <c:v>All Short Annual Return</c:v>
           </c:tx>
           <c:dLbls>
             <c:showLegendKey val="0"/>
@@ -194,6 +194,142 @@
           <c:idx val="3"/>
           <c:order val="3"/>
           <c:tx>
+            <c:v>All Short Beat</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Forward Beats Wide'!$B$2:$B$41</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Forward Beats Wide'!$F$2:$F$41</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Winner Long Annual Return</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Forward Beats Wide'!$B$2:$B$41</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Forward Beats Wide'!$G$2:$G$41</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>Winner Long Beat</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Forward Beats Wide'!$B$2:$B$41</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Forward Beats Wide'!$H$2:$H$41</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:v>Winner Short Annual Return</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Forward Beats Wide'!$B$2:$B$41</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Forward Beats Wide'!$I$2:$I$41</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:tx>
             <c:v>Winner Short Beat</c:v>
           </c:tx>
           <c:dLbls>
@@ -215,7 +351,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Forward Beats Wide'!$F$2:$F$41</c:f>
+              <c:f>'Forward Beats Wide'!$J$2:$J$41</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
@@ -361,7 +497,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3449e25658aa4a48"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra2e41f746c994f43"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -371,22 +507,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ForwardBeatWide" displayName="ForwardBeatWide" ref="A1:N41" headerRowCount="1">
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ForwardBeatWide" displayName="ForwardBeatWide" ref="A1:R41" headerRowCount="1">
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="Forward Quarters"/>
     <x:tableColumn id="2" name="Forward Years"/>
-    <x:tableColumn id="3" name="All Long Beat"/>
-    <x:tableColumn id="4" name="All Short Beat"/>
-    <x:tableColumn id="5" name="Winner Long Beat"/>
-    <x:tableColumn id="6" name="Winner Short Beat"/>
-    <x:tableColumn id="7" name="All Long Annual Return"/>
-    <x:tableColumn id="8" name="All Short Annual Return"/>
-    <x:tableColumn id="9" name="Winner Long Annual Return"/>
-    <x:tableColumn id="10" name="Winner Short Annual Return"/>
+    <x:tableColumn id="3" name="All Long Annual Return"/>
+    <x:tableColumn id="4" name="All Long Beat"/>
+    <x:tableColumn id="5" name="All Short Annual Return"/>
+    <x:tableColumn id="6" name="All Short Beat"/>
+    <x:tableColumn id="7" name="Winner Long Annual Return"/>
+    <x:tableColumn id="8" name="Winner Long Beat"/>
+    <x:tableColumn id="9" name="Winner Short Annual Return"/>
+    <x:tableColumn id="10" name="Winner Short Beat"/>
     <x:tableColumn id="11" name="All Long Count"/>
     <x:tableColumn id="12" name="All Short Count"/>
     <x:tableColumn id="13" name="Winner Long Count"/>
     <x:tableColumn id="14" name="Winner Short Count"/>
+    <x:tableColumn id="15" name="All Long Avg Years"/>
+    <x:tableColumn id="16" name="All Short Avg Years"/>
+    <x:tableColumn id="17" name="Winner Long Avg Years"/>
+    <x:tableColumn id="18" name="Winner Short Avg Years"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -589,22 +729,22 @@
   <x:cols>
     <x:col min="1" max="1" width="14.220000267028809" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.220000267028809" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="21.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="12.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15.4399995803833" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="15.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="14.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="14.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="17.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="17.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="15" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="15.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18.780000686645508" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -615,28 +755,28 @@
         <x:v>Forward Years</x:v>
       </x:c>
       <x:c r="C1" s="2" t="str">
+        <x:v>All Long Annual Return</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
         <x:v>All Long Beat</x:v>
       </x:c>
-      <x:c r="D1" s="2" t="str">
+      <x:c r="E1" s="2" t="str">
+        <x:v>All Short Annual Return</x:v>
+      </x:c>
+      <x:c r="F1" s="2" t="str">
         <x:v>All Short Beat</x:v>
       </x:c>
-      <x:c r="E1" s="2" t="str">
+      <x:c r="G1" s="2" t="str">
+        <x:v>Winner Long Annual Return</x:v>
+      </x:c>
+      <x:c r="H1" s="2" t="str">
         <x:v>Winner Long Beat</x:v>
       </x:c>
-      <x:c r="F1" s="2" t="str">
+      <x:c r="I1" s="2" t="str">
+        <x:v>Winner Short Annual Return</x:v>
+      </x:c>
+      <x:c r="J1" s="2" t="str">
         <x:v>Winner Short Beat</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>All Long Annual Return</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="str">
-        <x:v>All Short Annual Return</x:v>
-      </x:c>
-      <x:c r="I1" s="2" t="str">
-        <x:v>Winner Long Annual Return</x:v>
-      </x:c>
-      <x:c r="J1" s="2" t="str">
-        <x:v>Winner Short Annual Return</x:v>
       </x:c>
       <x:c r="K1" s="2" t="str">
         <x:v>All Long Count</x:v>
@@ -650,16 +790,16 @@
       <x:c r="N1" s="2" t="str">
         <x:v>Winner Short Count</x:v>
       </x:c>
-      <x:c r="O1" t="str">
+      <x:c r="O1" s="2" t="str">
         <x:v>All Long Avg Years</x:v>
       </x:c>
-      <x:c r="P1" t="str">
+      <x:c r="P1" s="2" t="str">
         <x:v>All Short Avg Years</x:v>
       </x:c>
-      <x:c r="Q1" t="str">
+      <x:c r="Q1" s="2" t="str">
         <x:v>Winner Long Avg Years</x:v>
       </x:c>
-      <x:c r="R1" t="str">
+      <x:c r="R1" s="2" t="str">
         <x:v>Winner Short Avg Years</x:v>
       </x:c>
     </x:row>
@@ -671,28 +811,28 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="C2" s="4" t="n">
+        <x:v>2.24823169</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="n">
         <x:v>2.09684963</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="n">
+      <x:c r="E2" s="4" t="n">
+        <x:v>0.25718404</x:v>
+      </x:c>
+      <x:c r="F2" s="4" t="n">
         <x:v>0.11016848</x:v>
       </x:c>
-      <x:c r="E2" s="4" t="n">
+      <x:c r="G2" s="4" t="n">
+        <x:v>13.251324810000002</x:v>
+      </x:c>
+      <x:c r="H2" s="4" t="n">
         <x:v>13.09311777</x:v>
       </x:c>
-      <x:c r="F2" s="4" t="n">
+      <x:c r="I2" s="4" t="n">
+        <x:v>0.36486362</x:v>
+      </x:c>
+      <x:c r="J2" s="4" t="n">
         <x:v>0.22472991</x:v>
-      </x:c>
-      <x:c r="G2" s="4" t="n">
-        <x:v>2.24823169</x:v>
-      </x:c>
-      <x:c r="H2" s="4" t="n">
-        <x:v>0.25718404</x:v>
-      </x:c>
-      <x:c r="I2" s="4" t="n">
-        <x:v>13.251324810000002</x:v>
-      </x:c>
-      <x:c r="J2" s="4" t="n">
-        <x:v>0.36486362</x:v>
       </x:c>
       <x:c r="K2" s="5" t="n">
         <x:v>2700</x:v>
@@ -727,28 +867,28 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="C3" s="4" t="n">
+        <x:v>0.39233845</x:v>
+      </x:c>
+      <x:c r="D3" s="4" t="n">
         <x:v>0.24759328</x:v>
       </x:c>
-      <x:c r="D3" s="4" t="n">
+      <x:c r="E3" s="4" t="n">
+        <x:v>0.05057315</x:v>
+      </x:c>
+      <x:c r="F3" s="4" t="n">
         <x:v>-0.07124741</x:v>
       </x:c>
-      <x:c r="E3" s="4" t="n">
+      <x:c r="G3" s="4" t="n">
+        <x:v>1.7213936699999999</x:v>
+      </x:c>
+      <x:c r="H3" s="4" t="n">
         <x:v>1.44225412</x:v>
       </x:c>
-      <x:c r="F3" s="4" t="n">
+      <x:c r="I3" s="4" t="n">
+        <x:v>0.11494623000000001</x:v>
+      </x:c>
+      <x:c r="J3" s="4" t="n">
         <x:v>0.02211067</x:v>
-      </x:c>
-      <x:c r="G3" s="4" t="n">
-        <x:v>0.39233845</x:v>
-      </x:c>
-      <x:c r="H3" s="4" t="n">
-        <x:v>0.05057315</x:v>
-      </x:c>
-      <x:c r="I3" s="4" t="n">
-        <x:v>1.7213936699999999</x:v>
-      </x:c>
-      <x:c r="J3" s="4" t="n">
-        <x:v>0.11494623000000001</x:v>
       </x:c>
       <x:c r="K3" s="5" t="n">
         <x:v>2700</x:v>
@@ -783,28 +923,28 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="C4" s="4" t="n">
+        <x:v>0.24742139999999999</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="n">
         <x:v>0.10602118</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="n">
+      <x:c r="E4" s="4" t="n">
+        <x:v>-0.0084732</x:v>
+      </x:c>
+      <x:c r="F4" s="4" t="n">
         <x:v>-0.12657378</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="n">
+      <x:c r="G4" s="4" t="n">
+        <x:v>1.1123960099999999</x:v>
+      </x:c>
+      <x:c r="H4" s="4" t="n">
         <x:v>0.7858886599999999</x:v>
       </x:c>
-      <x:c r="F4" s="4" t="n">
+      <x:c r="I4" s="4" t="n">
+        <x:v>0.06271391999999999</x:v>
+      </x:c>
+      <x:c r="J4" s="4" t="n">
         <x:v>-0.03363994</x:v>
-      </x:c>
-      <x:c r="G4" s="4" t="n">
-        <x:v>0.24742139999999999</x:v>
-      </x:c>
-      <x:c r="H4" s="4" t="n">
-        <x:v>-0.0084732</x:v>
-      </x:c>
-      <x:c r="I4" s="4" t="n">
-        <x:v>1.1123960099999999</x:v>
-      </x:c>
-      <x:c r="J4" s="4" t="n">
-        <x:v>0.06271391999999999</x:v>
       </x:c>
       <x:c r="K4" s="5" t="n">
         <x:v>2700</x:v>
@@ -839,28 +979,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
+        <x:v>0.17331331</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="n">
         <x:v>0.03237439</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="n">
+      <x:c r="E5" s="4" t="n">
+        <x:v>-0.025765660000000003</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="n">
         <x:v>-0.13809864</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="n">
+      <x:c r="G5" s="4" t="n">
+        <x:v>0.88268027</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="n">
         <x:v>0.5293873099999999</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="n">
+      <x:c r="I5" s="4" t="n">
+        <x:v>0.02088956</x:v>
+      </x:c>
+      <x:c r="J5" s="4" t="n">
         <x:v>-0.06953677</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="n">
-        <x:v>0.17331331</x:v>
-      </x:c>
-      <x:c r="H5" s="4" t="n">
-        <x:v>-0.025765660000000003</x:v>
-      </x:c>
-      <x:c r="I5" s="4" t="n">
-        <x:v>0.88268027</x:v>
-      </x:c>
-      <x:c r="J5" s="4" t="n">
-        <x:v>0.02088956</x:v>
       </x:c>
       <x:c r="K5" s="5" t="n">
         <x:v>2700</x:v>
@@ -895,28 +1035,28 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
+        <x:v>0.14220753</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="n">
         <x:v>0.00002065</x:v>
       </x:c>
-      <x:c r="D6" s="4" t="n">
+      <x:c r="E6" s="4" t="n">
+        <x:v>-0.03905462</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="n">
         <x:v>-0.15179735</x:v>
       </x:c>
-      <x:c r="E6" s="4" t="n">
+      <x:c r="G6" s="4" t="n">
+        <x:v>0.8366828</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="n">
         <x:v>0.43496505999999996</x:v>
       </x:c>
-      <x:c r="F6" s="4" t="n">
+      <x:c r="I6" s="4" t="n">
+        <x:v>0.01031148</x:v>
+      </x:c>
+      <x:c r="J6" s="4" t="n">
         <x:v>-0.08539844</x:v>
-      </x:c>
-      <x:c r="G6" s="4" t="n">
-        <x:v>0.14220753</x:v>
-      </x:c>
-      <x:c r="H6" s="4" t="n">
-        <x:v>-0.03905462</x:v>
-      </x:c>
-      <x:c r="I6" s="4" t="n">
-        <x:v>0.8366828</x:v>
-      </x:c>
-      <x:c r="J6" s="4" t="n">
-        <x:v>0.01031148</x:v>
       </x:c>
       <x:c r="K6" s="5" t="n">
         <x:v>2700</x:v>
@@ -951,28 +1091,28 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
+        <x:v>0.12556831000000002</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="n">
         <x:v>-0.019649859999999998</x:v>
       </x:c>
-      <x:c r="D7" s="4" t="n">
+      <x:c r="E7" s="4" t="n">
+        <x:v>-0.04314972</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="n">
         <x:v>-0.15583248</x:v>
       </x:c>
-      <x:c r="E7" s="4" t="n">
+      <x:c r="G7" s="4" t="n">
+        <x:v>0.7901467200000001</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="n">
         <x:v>0.3421975</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="n">
+      <x:c r="I7" s="4" t="n">
+        <x:v>0.01340144</x:v>
+      </x:c>
+      <x:c r="J7" s="4" t="n">
         <x:v>-0.07935047</x:v>
-      </x:c>
-      <x:c r="G7" s="4" t="n">
-        <x:v>0.12556831000000002</x:v>
-      </x:c>
-      <x:c r="H7" s="4" t="n">
-        <x:v>-0.04314972</x:v>
-      </x:c>
-      <x:c r="I7" s="4" t="n">
-        <x:v>0.7901467200000001</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="n">
-        <x:v>0.01340144</x:v>
       </x:c>
       <x:c r="K7" s="5" t="n">
         <x:v>2700</x:v>
@@ -1007,28 +1147,28 @@
         <x:v>1.75</x:v>
       </x:c>
       <x:c r="C8" s="4" t="n">
+        <x:v>0.11094817000000001</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="n">
         <x:v>-0.03743142</x:v>
       </x:c>
-      <x:c r="D8" s="4" t="n">
+      <x:c r="E8" s="4" t="n">
+        <x:v>-0.043118210000000004</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="n">
         <x:v>-0.15784511</x:v>
       </x:c>
-      <x:c r="E8" s="4" t="n">
+      <x:c r="G8" s="4" t="n">
+        <x:v>0.77526989</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="n">
         <x:v>0.30150953999999996</x:v>
       </x:c>
-      <x:c r="F8" s="4" t="n">
+      <x:c r="I8" s="4" t="n">
+        <x:v>-0.0031502200000000005</x:v>
+      </x:c>
+      <x:c r="J8" s="4" t="n">
         <x:v>-0.10121532999999999</x:v>
-      </x:c>
-      <x:c r="G8" s="4" t="n">
-        <x:v>0.11094817000000001</x:v>
-      </x:c>
-      <x:c r="H8" s="4" t="n">
-        <x:v>-0.043118210000000004</x:v>
-      </x:c>
-      <x:c r="I8" s="4" t="n">
-        <x:v>0.77526989</x:v>
-      </x:c>
-      <x:c r="J8" s="4" t="n">
-        <x:v>-0.0031502200000000005</x:v>
       </x:c>
       <x:c r="K8" s="5" t="n">
         <x:v>2700</x:v>
@@ -1063,28 +1203,28 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="4" t="n">
+        <x:v>0.10255887</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="n">
         <x:v>-0.047021610000000005</x:v>
       </x:c>
-      <x:c r="D9" s="4" t="n">
+      <x:c r="E9" s="4" t="n">
+        <x:v>-0.04105271</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="n">
         <x:v>-0.15668238</x:v>
       </x:c>
-      <x:c r="E9" s="4" t="n">
+      <x:c r="G9" s="4" t="n">
+        <x:v>0.78729079</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="n">
         <x:v>0.2870739</x:v>
       </x:c>
-      <x:c r="F9" s="4" t="n">
+      <x:c r="I9" s="4" t="n">
+        <x:v>0.0072936</x:v>
+      </x:c>
+      <x:c r="J9" s="4" t="n">
         <x:v>-0.0897294</x:v>
-      </x:c>
-      <x:c r="G9" s="4" t="n">
-        <x:v>0.10255887</x:v>
-      </x:c>
-      <x:c r="H9" s="4" t="n">
-        <x:v>-0.04105271</x:v>
-      </x:c>
-      <x:c r="I9" s="4" t="n">
-        <x:v>0.78729079</x:v>
-      </x:c>
-      <x:c r="J9" s="4" t="n">
-        <x:v>0.0072936</x:v>
       </x:c>
       <x:c r="K9" s="5" t="n">
         <x:v>2700</x:v>
@@ -1119,28 +1259,28 @@
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="C10" s="4" t="n">
+        <x:v>0.09505528999999999</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="n">
         <x:v>-0.05614853</x:v>
       </x:c>
-      <x:c r="D10" s="4" t="n">
+      <x:c r="E10" s="4" t="n">
+        <x:v>-0.04450799</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="n">
         <x:v>-0.16062328999999997</x:v>
       </x:c>
-      <x:c r="E10" s="4" t="n">
+      <x:c r="G10" s="4" t="n">
+        <x:v>0.76466207</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="n">
         <x:v>0.24808847</x:v>
       </x:c>
-      <x:c r="F10" s="4" t="n">
+      <x:c r="I10" s="4" t="n">
+        <x:v>0.00750408</x:v>
+      </x:c>
+      <x:c r="J10" s="4" t="n">
         <x:v>-0.08441209000000001</x:v>
-      </x:c>
-      <x:c r="G10" s="4" t="n">
-        <x:v>0.09505528999999999</x:v>
-      </x:c>
-      <x:c r="H10" s="4" t="n">
-        <x:v>-0.04450799</x:v>
-      </x:c>
-      <x:c r="I10" s="4" t="n">
-        <x:v>0.76466207</x:v>
-      </x:c>
-      <x:c r="J10" s="4" t="n">
-        <x:v>0.00750408</x:v>
       </x:c>
       <x:c r="K10" s="5" t="n">
         <x:v>2700</x:v>
@@ -1175,28 +1315,28 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="C11" s="4" t="n">
+        <x:v>0.09002432</x:v>
+      </x:c>
+      <x:c r="D11" s="4" t="n">
         <x:v>-0.06250963999999999</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="n">
+      <x:c r="E11" s="4" t="n">
+        <x:v>-0.04176406</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="n">
         <x:v>-0.15901998</x:v>
       </x:c>
-      <x:c r="E11" s="4" t="n">
+      <x:c r="G11" s="4" t="n">
+        <x:v>0.77425814</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="n">
         <x:v>0.24771844999999998</x:v>
       </x:c>
-      <x:c r="F11" s="4" t="n">
+      <x:c r="I11" s="4" t="n">
+        <x:v>0.01118937</x:v>
+      </x:c>
+      <x:c r="J11" s="4" t="n">
         <x:v>-0.08032844</x:v>
-      </x:c>
-      <x:c r="G11" s="4" t="n">
-        <x:v>0.09002432</x:v>
-      </x:c>
-      <x:c r="H11" s="4" t="n">
-        <x:v>-0.04176406</x:v>
-      </x:c>
-      <x:c r="I11" s="4" t="n">
-        <x:v>0.77425814</x:v>
-      </x:c>
-      <x:c r="J11" s="4" t="n">
-        <x:v>0.01118937</x:v>
       </x:c>
       <x:c r="K11" s="5" t="n">
         <x:v>2700</x:v>
@@ -1231,28 +1371,28 @@
         <x:v>2.75</x:v>
       </x:c>
       <x:c r="C12" s="4" t="n">
+        <x:v>0.09202362000000001</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="n">
         <x:v>-0.06244242</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="n">
+      <x:c r="E12" s="4" t="n">
+        <x:v>-0.037324989999999995</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="n">
         <x:v>-0.15588558</x:v>
       </x:c>
-      <x:c r="E12" s="4" t="n">
+      <x:c r="G12" s="4" t="n">
+        <x:v>0.77355458</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="n">
         <x:v>0.23519313</x:v>
       </x:c>
-      <x:c r="F12" s="4" t="n">
+      <x:c r="I12" s="4" t="n">
+        <x:v>0.02009764</x:v>
+      </x:c>
+      <x:c r="J12" s="4" t="n">
         <x:v>-0.06969739</x:v>
-      </x:c>
-      <x:c r="G12" s="4" t="n">
-        <x:v>0.09202362000000001</x:v>
-      </x:c>
-      <x:c r="H12" s="4" t="n">
-        <x:v>-0.037324989999999995</x:v>
-      </x:c>
-      <x:c r="I12" s="4" t="n">
-        <x:v>0.77355458</x:v>
-      </x:c>
-      <x:c r="J12" s="4" t="n">
-        <x:v>0.02009764</x:v>
       </x:c>
       <x:c r="K12" s="5" t="n">
         <x:v>2700</x:v>
@@ -1287,28 +1427,28 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="4" t="n">
+        <x:v>0.08932176</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="n">
         <x:v>-0.06673396000000001</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="n">
+      <x:c r="E13" s="4" t="n">
+        <x:v>-0.03847424</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="n">
         <x:v>-0.15814809</x:v>
       </x:c>
-      <x:c r="E13" s="4" t="n">
+      <x:c r="G13" s="4" t="n">
+        <x:v>0.75996892</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="n">
         <x:v>0.21080369000000002</x:v>
       </x:c>
-      <x:c r="F13" s="4" t="n">
+      <x:c r="I13" s="4" t="n">
+        <x:v>0.032826970000000004</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="n">
         <x:v>-0.05835143</x:v>
-      </x:c>
-      <x:c r="G13" s="4" t="n">
-        <x:v>0.08932176</x:v>
-      </x:c>
-      <x:c r="H13" s="4" t="n">
-        <x:v>-0.03847424</x:v>
-      </x:c>
-      <x:c r="I13" s="4" t="n">
-        <x:v>0.75996892</x:v>
-      </x:c>
-      <x:c r="J13" s="4" t="n">
-        <x:v>0.032826970000000004</x:v>
       </x:c>
       <x:c r="K13" s="5" t="n">
         <x:v>2700</x:v>
@@ -1343,28 +1483,28 @@
         <x:v>3.25</x:v>
       </x:c>
       <x:c r="C14" s="4" t="n">
+        <x:v>0.08613728999999999</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="n">
         <x:v>-0.07138751</x:v>
       </x:c>
-      <x:c r="D14" s="4" t="n">
+      <x:c r="E14" s="4" t="n">
+        <x:v>-0.03398754</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="n">
         <x:v>-0.15493949</x:v>
       </x:c>
-      <x:c r="E14" s="4" t="n">
+      <x:c r="G14" s="4" t="n">
+        <x:v>0.7610820300000001</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="n">
         <x:v>0.20091024999999998</x:v>
       </x:c>
-      <x:c r="F14" s="4" t="n">
+      <x:c r="I14" s="4" t="n">
+        <x:v>0.0257943</x:v>
+      </x:c>
+      <x:c r="J14" s="4" t="n">
         <x:v>-0.06947901</x:v>
-      </x:c>
-      <x:c r="G14" s="4" t="n">
-        <x:v>0.08613728999999999</x:v>
-      </x:c>
-      <x:c r="H14" s="4" t="n">
-        <x:v>-0.03398754</x:v>
-      </x:c>
-      <x:c r="I14" s="4" t="n">
-        <x:v>0.7610820300000001</x:v>
-      </x:c>
-      <x:c r="J14" s="4" t="n">
-        <x:v>0.0257943</x:v>
       </x:c>
       <x:c r="K14" s="5" t="n">
         <x:v>2700</x:v>
@@ -1399,28 +1539,28 @@
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="C15" s="4" t="n">
+        <x:v>0.08456089</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="n">
         <x:v>-0.07296469</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="n">
+      <x:c r="E15" s="4" t="n">
+        <x:v>-0.032100529999999995</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="n">
         <x:v>-0.15410417</x:v>
       </x:c>
-      <x:c r="E15" s="4" t="n">
+      <x:c r="G15" s="4" t="n">
+        <x:v>0.7530800999999999</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="n">
         <x:v>0.18524174999999998</x:v>
       </x:c>
-      <x:c r="F15" s="4" t="n">
+      <x:c r="I15" s="4" t="n">
+        <x:v>0.023804759999999998</x:v>
+      </x:c>
+      <x:c r="J15" s="4" t="n">
         <x:v>-0.07203282</x:v>
-      </x:c>
-      <x:c r="G15" s="4" t="n">
-        <x:v>0.08456089</x:v>
-      </x:c>
-      <x:c r="H15" s="4" t="n">
-        <x:v>-0.032100529999999995</x:v>
-      </x:c>
-      <x:c r="I15" s="4" t="n">
-        <x:v>0.7530800999999999</x:v>
-      </x:c>
-      <x:c r="J15" s="4" t="n">
-        <x:v>0.023804759999999998</x:v>
       </x:c>
       <x:c r="K15" s="5" t="n">
         <x:v>2700</x:v>
@@ -1455,28 +1595,28 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="C16" s="4" t="n">
+        <x:v>0.08314926</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="n">
         <x:v>-0.07487475</x:v>
       </x:c>
-      <x:c r="D16" s="4" t="n">
+      <x:c r="E16" s="4" t="n">
+        <x:v>-0.03220619</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="n">
         <x:v>-0.15546027</x:v>
       </x:c>
-      <x:c r="E16" s="4" t="n">
+      <x:c r="G16" s="4" t="n">
+        <x:v>0.73816616</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="n">
         <x:v>0.16269943</x:v>
       </x:c>
-      <x:c r="F16" s="4" t="n">
+      <x:c r="I16" s="4" t="n">
+        <x:v>-0.0046911900000000005</x:v>
+      </x:c>
+      <x:c r="J16" s="4" t="n">
         <x:v>-0.10291204000000001</x:v>
-      </x:c>
-      <x:c r="G16" s="4" t="n">
-        <x:v>0.08314926</x:v>
-      </x:c>
-      <x:c r="H16" s="4" t="n">
-        <x:v>-0.03220619</x:v>
-      </x:c>
-      <x:c r="I16" s="4" t="n">
-        <x:v>0.73816616</x:v>
-      </x:c>
-      <x:c r="J16" s="4" t="n">
-        <x:v>-0.0046911900000000005</x:v>
       </x:c>
       <x:c r="K16" s="5" t="n">
         <x:v>2700</x:v>
@@ -1511,28 +1651,28 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C17" s="4" t="n">
+        <x:v>0.08002729</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="n">
         <x:v>-0.07866987</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="n">
+      <x:c r="E17" s="4" t="n">
+        <x:v>-0.02629399</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="n">
         <x:v>-0.15016864</x:v>
       </x:c>
-      <x:c r="E17" s="4" t="n">
+      <x:c r="G17" s="4" t="n">
+        <x:v>0.73486666</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="n">
         <x:v>0.14919665000000001</x:v>
       </x:c>
-      <x:c r="F17" s="4" t="n">
+      <x:c r="I17" s="4" t="n">
+        <x:v>0.01501994</x:v>
+      </x:c>
+      <x:c r="J17" s="4" t="n">
         <x:v>-0.08682121999999999</x:v>
-      </x:c>
-      <x:c r="G17" s="4" t="n">
-        <x:v>0.08002729</x:v>
-      </x:c>
-      <x:c r="H17" s="4" t="n">
-        <x:v>-0.02629399</x:v>
-      </x:c>
-      <x:c r="I17" s="4" t="n">
-        <x:v>0.73486666</x:v>
-      </x:c>
-      <x:c r="J17" s="4" t="n">
-        <x:v>0.01501994</x:v>
       </x:c>
       <x:c r="K17" s="5" t="n">
         <x:v>2700</x:v>
@@ -1567,28 +1707,28 @@
         <x:v>4.25</x:v>
       </x:c>
       <x:c r="C18" s="4" t="n">
+        <x:v>0.07890989</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="n">
         <x:v>-0.0795706</x:v>
       </x:c>
-      <x:c r="D18" s="4" t="n">
+      <x:c r="E18" s="4" t="n">
+        <x:v>-0.02630046</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="n">
         <x:v>-0.15145261</x:v>
       </x:c>
-      <x:c r="E18" s="4" t="n">
+      <x:c r="G18" s="4" t="n">
+        <x:v>0.71473337</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="n">
         <x:v>0.12224317</x:v>
       </x:c>
-      <x:c r="F18" s="4" t="n">
+      <x:c r="I18" s="4" t="n">
+        <x:v>-0.00227935</x:v>
+      </x:c>
+      <x:c r="J18" s="4" t="n">
         <x:v>-0.11122488000000001</x:v>
-      </x:c>
-      <x:c r="G18" s="4" t="n">
-        <x:v>0.07890989</x:v>
-      </x:c>
-      <x:c r="H18" s="4" t="n">
-        <x:v>-0.02630046</x:v>
-      </x:c>
-      <x:c r="I18" s="4" t="n">
-        <x:v>0.71473337</x:v>
-      </x:c>
-      <x:c r="J18" s="4" t="n">
-        <x:v>-0.00227935</x:v>
       </x:c>
       <x:c r="K18" s="5" t="n">
         <x:v>2700</x:v>
@@ -1623,28 +1763,28 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="C19" s="4" t="n">
+        <x:v>0.07733747</x:v>
+      </x:c>
+      <x:c r="D19" s="4" t="n">
         <x:v>-0.08127632</x:v>
       </x:c>
-      <x:c r="D19" s="4" t="n">
+      <x:c r="E19" s="4" t="n">
+        <x:v>-0.024729619999999997</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="n">
         <x:v>-0.15081706</x:v>
       </x:c>
-      <x:c r="E19" s="4" t="n">
+      <x:c r="G19" s="4" t="n">
+        <x:v>0.70834075</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="n">
         <x:v>0.1099639</x:v>
       </x:c>
-      <x:c r="F19" s="4" t="n">
+      <x:c r="I19" s="4" t="n">
+        <x:v>-0.0019506100000000002</x:v>
+      </x:c>
+      <x:c r="J19" s="4" t="n">
         <x:v>-0.1137833</x:v>
-      </x:c>
-      <x:c r="G19" s="4" t="n">
-        <x:v>0.07733747</x:v>
-      </x:c>
-      <x:c r="H19" s="4" t="n">
-        <x:v>-0.024729619999999997</x:v>
-      </x:c>
-      <x:c r="I19" s="4" t="n">
-        <x:v>0.70834075</x:v>
-      </x:c>
-      <x:c r="J19" s="4" t="n">
-        <x:v>-0.0019506100000000002</x:v>
       </x:c>
       <x:c r="K19" s="5" t="n">
         <x:v>2700</x:v>
@@ -1679,28 +1819,28 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="C20" s="4" t="n">
+        <x:v>0.07675477</x:v>
+      </x:c>
+      <x:c r="D20" s="4" t="n">
         <x:v>-0.08175044</x:v>
       </x:c>
-      <x:c r="D20" s="4" t="n">
+      <x:c r="E20" s="4" t="n">
+        <x:v>-0.02104819</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="n">
         <x:v>-0.14733241</x:v>
       </x:c>
-      <x:c r="E20" s="4" t="n">
+      <x:c r="G20" s="4" t="n">
+        <x:v>0.71559037</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="n">
         <x:v>0.11277879</x:v>
       </x:c>
-      <x:c r="F20" s="4" t="n">
+      <x:c r="I20" s="4" t="n">
+        <x:v>0.0114879</x:v>
+      </x:c>
+      <x:c r="J20" s="4" t="n">
         <x:v>-0.09378943</x:v>
-      </x:c>
-      <x:c r="G20" s="4" t="n">
-        <x:v>0.07675477</x:v>
-      </x:c>
-      <x:c r="H20" s="4" t="n">
-        <x:v>-0.02104819</x:v>
-      </x:c>
-      <x:c r="I20" s="4" t="n">
-        <x:v>0.71559037</x:v>
-      </x:c>
-      <x:c r="J20" s="4" t="n">
-        <x:v>0.0114879</x:v>
       </x:c>
       <x:c r="K20" s="5" t="n">
         <x:v>2700</x:v>
@@ -1735,28 +1875,28 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="4" t="n">
+        <x:v>0.0758809</x:v>
+      </x:c>
+      <x:c r="D21" s="4" t="n">
         <x:v>-0.08194342</x:v>
       </x:c>
-      <x:c r="D21" s="4" t="n">
+      <x:c r="E21" s="4" t="n">
+        <x:v>-0.01856386</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="n">
         <x:v>-0.1447298</x:v>
       </x:c>
-      <x:c r="E21" s="4" t="n">
+      <x:c r="G21" s="4" t="n">
+        <x:v>0.71062455</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="n">
         <x:v>0.10344272</x:v>
       </x:c>
-      <x:c r="F21" s="4" t="n">
+      <x:c r="I21" s="4" t="n">
+        <x:v>0.00246159</x:v>
+      </x:c>
+      <x:c r="J21" s="4" t="n">
         <x:v>-0.10493866</x:v>
-      </x:c>
-      <x:c r="G21" s="4" t="n">
-        <x:v>0.0758809</x:v>
-      </x:c>
-      <x:c r="H21" s="4" t="n">
-        <x:v>-0.01856386</x:v>
-      </x:c>
-      <x:c r="I21" s="4" t="n">
-        <x:v>0.71062455</x:v>
-      </x:c>
-      <x:c r="J21" s="4" t="n">
-        <x:v>0.00246159</x:v>
       </x:c>
       <x:c r="K21" s="5" t="n">
         <x:v>2700</x:v>
@@ -1791,28 +1931,28 @@
         <x:v>5.25</x:v>
       </x:c>
       <x:c r="C22" s="4" t="n">
+        <x:v>0.07514735</x:v>
+      </x:c>
+      <x:c r="D22" s="4" t="n">
         <x:v>-0.08276863000000001</x:v>
       </x:c>
-      <x:c r="D22" s="4" t="n">
+      <x:c r="E22" s="4" t="n">
+        <x:v>-0.01741189</x:v>
+      </x:c>
+      <x:c r="F22" s="4" t="n">
         <x:v>-0.14502652</x:v>
       </x:c>
-      <x:c r="E22" s="4" t="n">
+      <x:c r="G22" s="4" t="n">
+        <x:v>0.7134843700000001</x:v>
+      </x:c>
+      <x:c r="H22" s="4" t="n">
         <x:v>0.10237738</x:v>
       </x:c>
-      <x:c r="F22" s="4" t="n">
+      <x:c r="I22" s="4" t="n">
+        <x:v>0.00423328</x:v>
+      </x:c>
+      <x:c r="J22" s="4" t="n">
         <x:v>-0.10697424</x:v>
-      </x:c>
-      <x:c r="G22" s="4" t="n">
-        <x:v>0.07514735</x:v>
-      </x:c>
-      <x:c r="H22" s="4" t="n">
-        <x:v>-0.01741189</x:v>
-      </x:c>
-      <x:c r="I22" s="4" t="n">
-        <x:v>0.7134843700000001</x:v>
-      </x:c>
-      <x:c r="J22" s="4" t="n">
-        <x:v>0.00423328</x:v>
       </x:c>
       <x:c r="K22" s="5" t="n">
         <x:v>2700</x:v>
@@ -1847,28 +1987,28 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="C23" s="4" t="n">
+        <x:v>0.07401562</x:v>
+      </x:c>
+      <x:c r="D23" s="4" t="n">
         <x:v>-0.08444378000000001</x:v>
       </x:c>
-      <x:c r="D23" s="4" t="n">
+      <x:c r="E23" s="4" t="n">
+        <x:v>-0.016525579999999998</x:v>
+      </x:c>
+      <x:c r="F23" s="4" t="n">
         <x:v>-0.14541458000000002</x:v>
       </x:c>
-      <x:c r="E23" s="4" t="n">
+      <x:c r="G23" s="4" t="n">
+        <x:v>0.71274644</x:v>
+      </x:c>
+      <x:c r="H23" s="4" t="n">
         <x:v>0.09812398</x:v>
       </x:c>
-      <x:c r="F23" s="4" t="n">
+      <x:c r="I23" s="4" t="n">
+        <x:v>0.00000193</x:v>
+      </x:c>
+      <x:c r="J23" s="4" t="n">
         <x:v>-0.11284015</x:v>
-      </x:c>
-      <x:c r="G23" s="4" t="n">
-        <x:v>0.07401562</x:v>
-      </x:c>
-      <x:c r="H23" s="4" t="n">
-        <x:v>-0.016525579999999998</x:v>
-      </x:c>
-      <x:c r="I23" s="4" t="n">
-        <x:v>0.71274644</x:v>
-      </x:c>
-      <x:c r="J23" s="4" t="n">
-        <x:v>0.00000193</x:v>
       </x:c>
       <x:c r="K23" s="5" t="n">
         <x:v>2700</x:v>
@@ -1903,28 +2043,28 @@
         <x:v>5.75</x:v>
       </x:c>
       <x:c r="C24" s="4" t="n">
+        <x:v>0.07311567000000001</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="n">
         <x:v>-0.08521266000000001</x:v>
       </x:c>
-      <x:c r="D24" s="4" t="n">
+      <x:c r="E24" s="4" t="n">
+        <x:v>-0.015606580000000002</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="n">
         <x:v>-0.14551841</x:v>
       </x:c>
-      <x:c r="E24" s="4" t="n">
+      <x:c r="G24" s="4" t="n">
+        <x:v>0.71128163</x:v>
+      </x:c>
+      <x:c r="H24" s="4" t="n">
         <x:v>0.09152996</x:v>
       </x:c>
-      <x:c r="F24" s="4" t="n">
+      <x:c r="I24" s="4" t="n">
+        <x:v>0.00748991</x:v>
+      </x:c>
+      <x:c r="J24" s="4" t="n">
         <x:v>-0.10432454999999999</x:v>
-      </x:c>
-      <x:c r="G24" s="4" t="n">
-        <x:v>0.07311567000000001</x:v>
-      </x:c>
-      <x:c r="H24" s="4" t="n">
-        <x:v>-0.015606580000000002</x:v>
-      </x:c>
-      <x:c r="I24" s="4" t="n">
-        <x:v>0.71128163</x:v>
-      </x:c>
-      <x:c r="J24" s="4" t="n">
-        <x:v>0.00748991</x:v>
       </x:c>
       <x:c r="K24" s="5" t="n">
         <x:v>2700</x:v>
@@ -1959,28 +2099,28 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C25" s="4" t="n">
+        <x:v>0.07292462000000001</x:v>
+      </x:c>
+      <x:c r="D25" s="4" t="n">
         <x:v>-0.08517493999999999</x:v>
       </x:c>
-      <x:c r="D25" s="4" t="n">
+      <x:c r="E25" s="4" t="n">
+        <x:v>-0.015038339999999999</x:v>
+      </x:c>
+      <x:c r="F25" s="4" t="n">
         <x:v>-0.145875</x:v>
       </x:c>
-      <x:c r="E25" s="4" t="n">
+      <x:c r="G25" s="4" t="n">
+        <x:v>0.7140234599999999</x:v>
+      </x:c>
+      <x:c r="H25" s="4" t="n">
         <x:v>0.09248946999999999</x:v>
       </x:c>
-      <x:c r="F25" s="4" t="n">
+      <x:c r="I25" s="4" t="n">
+        <x:v>-0.00367682</x:v>
+      </x:c>
+      <x:c r="J25" s="4" t="n">
         <x:v>-0.11794807</x:v>
-      </x:c>
-      <x:c r="G25" s="4" t="n">
-        <x:v>0.07292462000000001</x:v>
-      </x:c>
-      <x:c r="H25" s="4" t="n">
-        <x:v>-0.015038339999999999</x:v>
-      </x:c>
-      <x:c r="I25" s="4" t="n">
-        <x:v>0.7140234599999999</x:v>
-      </x:c>
-      <x:c r="J25" s="4" t="n">
-        <x:v>-0.00367682</x:v>
       </x:c>
       <x:c r="K25" s="5" t="n">
         <x:v>2700</x:v>
@@ -2015,28 +2155,28 @@
         <x:v>6.25</x:v>
       </x:c>
       <x:c r="C26" s="4" t="n">
+        <x:v>0.07242833</x:v>
+      </x:c>
+      <x:c r="D26" s="4" t="n">
         <x:v>-0.08581214</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="n">
+      <x:c r="E26" s="4" t="n">
+        <x:v>-0.013203769999999998</x:v>
+      </x:c>
+      <x:c r="F26" s="4" t="n">
         <x:v>-0.14449087</x:v>
       </x:c>
-      <x:c r="E26" s="4" t="n">
+      <x:c r="G26" s="4" t="n">
+        <x:v>0.71447977</x:v>
+      </x:c>
+      <x:c r="H26" s="4" t="n">
         <x:v>0.09077088</x:v>
       </x:c>
-      <x:c r="F26" s="4" t="n">
+      <x:c r="I26" s="4" t="n">
+        <x:v>0.00370828</x:v>
+      </x:c>
+      <x:c r="J26" s="4" t="n">
         <x:v>-0.11050867</x:v>
-      </x:c>
-      <x:c r="G26" s="4" t="n">
-        <x:v>0.07242833</x:v>
-      </x:c>
-      <x:c r="H26" s="4" t="n">
-        <x:v>-0.013203769999999998</x:v>
-      </x:c>
-      <x:c r="I26" s="4" t="n">
-        <x:v>0.71447977</x:v>
-      </x:c>
-      <x:c r="J26" s="4" t="n">
-        <x:v>0.00370828</x:v>
       </x:c>
       <x:c r="K26" s="5" t="n">
         <x:v>2700</x:v>
@@ -2071,28 +2211,28 @@
         <x:v>6.5</x:v>
       </x:c>
       <x:c r="C27" s="4" t="n">
+        <x:v>0.07244373</x:v>
+      </x:c>
+      <x:c r="D27" s="4" t="n">
         <x:v>-0.08565292</x:v>
       </x:c>
-      <x:c r="D27" s="4" t="n">
+      <x:c r="E27" s="4" t="n">
+        <x:v>-0.01156242</x:v>
+      </x:c>
+      <x:c r="F27" s="4" t="n">
         <x:v>-0.14310118</x:v>
       </x:c>
-      <x:c r="E27" s="4" t="n">
+      <x:c r="G27" s="4" t="n">
+        <x:v>0.71410273</x:v>
+      </x:c>
+      <x:c r="H27" s="4" t="n">
         <x:v>0.08589905999999999</x:v>
       </x:c>
-      <x:c r="F27" s="4" t="n">
+      <x:c r="I27" s="4" t="n">
+        <x:v>-0.0025236300000000002</x:v>
+      </x:c>
+      <x:c r="J27" s="4" t="n">
         <x:v>-0.11914403999999999</x:v>
-      </x:c>
-      <x:c r="G27" s="4" t="n">
-        <x:v>0.07244373</x:v>
-      </x:c>
-      <x:c r="H27" s="4" t="n">
-        <x:v>-0.01156242</x:v>
-      </x:c>
-      <x:c r="I27" s="4" t="n">
-        <x:v>0.71410273</x:v>
-      </x:c>
-      <x:c r="J27" s="4" t="n">
-        <x:v>-0.0025236300000000002</x:v>
       </x:c>
       <x:c r="K27" s="5" t="n">
         <x:v>2700</x:v>
@@ -2127,28 +2267,28 @@
         <x:v>6.75</x:v>
       </x:c>
       <x:c r="C28" s="4" t="n">
+        <x:v>0.07197154</x:v>
+      </x:c>
+      <x:c r="D28" s="4" t="n">
         <x:v>-0.08625392</x:v>
       </x:c>
-      <x:c r="D28" s="4" t="n">
+      <x:c r="E28" s="4" t="n">
+        <x:v>-0.01052451</x:v>
+      </x:c>
+      <x:c r="F28" s="4" t="n">
         <x:v>-0.14275758</x:v>
       </x:c>
-      <x:c r="E28" s="4" t="n">
+      <x:c r="G28" s="4" t="n">
+        <x:v>0.71277247</x:v>
+      </x:c>
+      <x:c r="H28" s="4" t="n">
         <x:v>0.08106661000000001</x:v>
       </x:c>
-      <x:c r="F28" s="4" t="n">
+      <x:c r="I28" s="4" t="n">
+        <x:v>0.00473786</x:v>
+      </x:c>
+      <x:c r="J28" s="4" t="n">
         <x:v>-0.11286602999999999</x:v>
-      </x:c>
-      <x:c r="G28" s="4" t="n">
-        <x:v>0.07197154</x:v>
-      </x:c>
-      <x:c r="H28" s="4" t="n">
-        <x:v>-0.01052451</x:v>
-      </x:c>
-      <x:c r="I28" s="4" t="n">
-        <x:v>0.71277247</x:v>
-      </x:c>
-      <x:c r="J28" s="4" t="n">
-        <x:v>0.00473786</x:v>
       </x:c>
       <x:c r="K28" s="5" t="n">
         <x:v>2700</x:v>
@@ -2183,28 +2323,28 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C29" s="4" t="n">
+        <x:v>0.07099008000000001</x:v>
+      </x:c>
+      <x:c r="D29" s="4" t="n">
         <x:v>-0.08724453</x:v>
       </x:c>
-      <x:c r="D29" s="4" t="n">
+      <x:c r="E29" s="4" t="n">
+        <x:v>-0.01057723</x:v>
+      </x:c>
+      <x:c r="F29" s="4" t="n">
         <x:v>-0.14385314</x:v>
       </x:c>
-      <x:c r="E29" s="4" t="n">
+      <x:c r="G29" s="4" t="n">
+        <x:v>0.71119622</x:v>
+      </x:c>
+      <x:c r="H29" s="4" t="n">
         <x:v>0.07626068</x:v>
       </x:c>
-      <x:c r="F29" s="4" t="n">
+      <x:c r="I29" s="4" t="n">
+        <x:v>-0.00876789</x:v>
+      </x:c>
+      <x:c r="J29" s="4" t="n">
         <x:v>-0.133162</x:v>
-      </x:c>
-      <x:c r="G29" s="4" t="n">
-        <x:v>0.07099008000000001</x:v>
-      </x:c>
-      <x:c r="H29" s="4" t="n">
-        <x:v>-0.01057723</x:v>
-      </x:c>
-      <x:c r="I29" s="4" t="n">
-        <x:v>0.71119622</x:v>
-      </x:c>
-      <x:c r="J29" s="4" t="n">
-        <x:v>-0.00876789</x:v>
       </x:c>
       <x:c r="K29" s="5" t="n">
         <x:v>2700</x:v>
@@ -2239,28 +2379,28 @@
         <x:v>7.25</x:v>
       </x:c>
       <x:c r="C30" s="4" t="n">
+        <x:v>0.07098623</x:v>
+      </x:c>
+      <x:c r="D30" s="4" t="n">
         <x:v>-0.08675118</x:v>
       </x:c>
-      <x:c r="D30" s="4" t="n">
+      <x:c r="E30" s="4" t="n">
+        <x:v>-0.00840723</x:v>
+      </x:c>
+      <x:c r="F30" s="4" t="n">
         <x:v>-0.14204597</x:v>
       </x:c>
-      <x:c r="E30" s="4" t="n">
+      <x:c r="G30" s="4" t="n">
+        <x:v>0.70595303</x:v>
+      </x:c>
+      <x:c r="H30" s="4" t="n">
         <x:v>0.07025065999999999</x:v>
       </x:c>
-      <x:c r="F30" s="4" t="n">
+      <x:c r="I30" s="4" t="n">
+        <x:v>0.0120945</x:v>
+      </x:c>
+      <x:c r="J30" s="4" t="n">
         <x:v>-0.10940025</x:v>
-      </x:c>
-      <x:c r="G30" s="4" t="n">
-        <x:v>0.07098623</x:v>
-      </x:c>
-      <x:c r="H30" s="4" t="n">
-        <x:v>-0.00840723</x:v>
-      </x:c>
-      <x:c r="I30" s="4" t="n">
-        <x:v>0.70595303</x:v>
-      </x:c>
-      <x:c r="J30" s="4" t="n">
-        <x:v>0.0120945</x:v>
       </x:c>
       <x:c r="K30" s="5" t="n">
         <x:v>2700</x:v>
@@ -2295,28 +2435,28 @@
         <x:v>7.5</x:v>
       </x:c>
       <x:c r="C31" s="4" t="n">
+        <x:v>0.07061128</x:v>
+      </x:c>
+      <x:c r="D31" s="4" t="n">
         <x:v>-0.08724768</x:v>
       </x:c>
-      <x:c r="D31" s="4" t="n">
+      <x:c r="E31" s="4" t="n">
+        <x:v>-0.00827957</x:v>
+      </x:c>
+      <x:c r="F31" s="4" t="n">
         <x:v>-0.14238759</x:v>
       </x:c>
-      <x:c r="E31" s="4" t="n">
+      <x:c r="G31" s="4" t="n">
+        <x:v>0.7043785300000001</x:v>
+      </x:c>
+      <x:c r="H31" s="4" t="n">
         <x:v>0.06497098</x:v>
       </x:c>
-      <x:c r="F31" s="4" t="n">
+      <x:c r="I31" s="4" t="n">
+        <x:v>0.00368604</x:v>
+      </x:c>
+      <x:c r="J31" s="4" t="n">
         <x:v>-0.11961812</x:v>
-      </x:c>
-      <x:c r="G31" s="4" t="n">
-        <x:v>0.07061128</x:v>
-      </x:c>
-      <x:c r="H31" s="4" t="n">
-        <x:v>-0.00827957</x:v>
-      </x:c>
-      <x:c r="I31" s="4" t="n">
-        <x:v>0.7043785300000001</x:v>
-      </x:c>
-      <x:c r="J31" s="4" t="n">
-        <x:v>0.00368604</x:v>
       </x:c>
       <x:c r="K31" s="5" t="n">
         <x:v>2700</x:v>
@@ -2351,28 +2491,28 @@
         <x:v>7.75</x:v>
       </x:c>
       <x:c r="C32" s="4" t="n">
+        <x:v>0.06992869</x:v>
+      </x:c>
+      <x:c r="D32" s="4" t="n">
         <x:v>-0.08771672999999999</x:v>
       </x:c>
-      <x:c r="D32" s="4" t="n">
+      <x:c r="E32" s="4" t="n">
+        <x:v>-0.00995782</x:v>
+      </x:c>
+      <x:c r="F32" s="4" t="n">
         <x:v>-0.14565065</x:v>
       </x:c>
-      <x:c r="E32" s="4" t="n">
+      <x:c r="G32" s="4" t="n">
+        <x:v>0.7050791099999999</x:v>
+      </x:c>
+      <x:c r="H32" s="4" t="n">
         <x:v>0.06390123</x:v>
       </x:c>
-      <x:c r="F32" s="4" t="n">
+      <x:c r="I32" s="4" t="n">
+        <x:v>0.00901543</x:v>
+      </x:c>
+      <x:c r="J32" s="4" t="n">
         <x:v>-0.11825642</x:v>
-      </x:c>
-      <x:c r="G32" s="4" t="n">
-        <x:v>0.06992869</x:v>
-      </x:c>
-      <x:c r="H32" s="4" t="n">
-        <x:v>-0.00995782</x:v>
-      </x:c>
-      <x:c r="I32" s="4" t="n">
-        <x:v>0.7050791099999999</x:v>
-      </x:c>
-      <x:c r="J32" s="4" t="n">
-        <x:v>0.00901543</x:v>
       </x:c>
       <x:c r="K32" s="5" t="n">
         <x:v>2700</x:v>
@@ -2407,28 +2547,28 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="4" t="n">
+        <x:v>0.07037093</x:v>
+      </x:c>
+      <x:c r="D33" s="4" t="n">
         <x:v>-0.08746663</x:v>
       </x:c>
-      <x:c r="D33" s="4" t="n">
+      <x:c r="E33" s="4" t="n">
+        <x:v>-0.00870937</x:v>
+      </x:c>
+      <x:c r="F33" s="4" t="n">
         <x:v>-0.14435053</x:v>
       </x:c>
-      <x:c r="E33" s="4" t="n">
+      <x:c r="G33" s="4" t="n">
+        <x:v>0.7061083100000001</x:v>
+      </x:c>
+      <x:c r="H33" s="4" t="n">
         <x:v>0.062249679999999995</x:v>
       </x:c>
-      <x:c r="F33" s="4" t="n">
+      <x:c r="I33" s="4" t="n">
+        <x:v>0.007530909999999999</x:v>
+      </x:c>
+      <x:c r="J33" s="4" t="n">
         <x:v>-0.12116211</x:v>
-      </x:c>
-      <x:c r="G33" s="4" t="n">
-        <x:v>0.07037093</x:v>
-      </x:c>
-      <x:c r="H33" s="4" t="n">
-        <x:v>-0.00870937</x:v>
-      </x:c>
-      <x:c r="I33" s="4" t="n">
-        <x:v>0.7061083100000001</x:v>
-      </x:c>
-      <x:c r="J33" s="4" t="n">
-        <x:v>0.007530909999999999</x:v>
       </x:c>
       <x:c r="K33" s="5" t="n">
         <x:v>2700</x:v>
@@ -2463,28 +2603,28 @@
         <x:v>8.25</x:v>
       </x:c>
       <x:c r="C34" s="4" t="n">
+        <x:v>0.0703958</x:v>
+      </x:c>
+      <x:c r="D34" s="4" t="n">
         <x:v>-0.08753875000000001</x:v>
       </x:c>
-      <x:c r="D34" s="4" t="n">
+      <x:c r="E34" s="4" t="n">
+        <x:v>-0.00609143</x:v>
+      </x:c>
+      <x:c r="F34" s="4" t="n">
         <x:v>-0.14165192</x:v>
       </x:c>
-      <x:c r="E34" s="4" t="n">
+      <x:c r="G34" s="4" t="n">
+        <x:v>0.70355215</x:v>
+      </x:c>
+      <x:c r="H34" s="4" t="n">
         <x:v>0.05706486</x:v>
       </x:c>
-      <x:c r="F34" s="4" t="n">
+      <x:c r="I34" s="4" t="n">
+        <x:v>0.01298729</x:v>
+      </x:c>
+      <x:c r="J34" s="4" t="n">
         <x:v>-0.11531568</x:v>
-      </x:c>
-      <x:c r="G34" s="4" t="n">
-        <x:v>0.0703958</x:v>
-      </x:c>
-      <x:c r="H34" s="4" t="n">
-        <x:v>-0.00609143</x:v>
-      </x:c>
-      <x:c r="I34" s="4" t="n">
-        <x:v>0.70355215</x:v>
-      </x:c>
-      <x:c r="J34" s="4" t="n">
-        <x:v>0.01298729</x:v>
       </x:c>
       <x:c r="K34" s="5" t="n">
         <x:v>2700</x:v>
@@ -2519,28 +2659,28 @@
         <x:v>8.5</x:v>
       </x:c>
       <x:c r="C35" s="4" t="n">
+        <x:v>0.06997463</x:v>
+      </x:c>
+      <x:c r="D35" s="4" t="n">
         <x:v>-0.08779089000000001</x:v>
       </x:c>
-      <x:c r="D35" s="4" t="n">
+      <x:c r="E35" s="4" t="n">
+        <x:v>-0.00595619</x:v>
+      </x:c>
+      <x:c r="F35" s="4" t="n">
         <x:v>-0.14188335</x:v>
       </x:c>
-      <x:c r="E35" s="4" t="n">
+      <x:c r="G35" s="4" t="n">
+        <x:v>0.70160807</x:v>
+      </x:c>
+      <x:c r="H35" s="4" t="n">
         <x:v>0.05149625</x:v>
       </x:c>
-      <x:c r="F35" s="4" t="n">
+      <x:c r="I35" s="4" t="n">
+        <x:v>0.01430439</x:v>
+      </x:c>
+      <x:c r="J35" s="4" t="n">
         <x:v>-0.11499204</x:v>
-      </x:c>
-      <x:c r="G35" s="4" t="n">
-        <x:v>0.06997463</x:v>
-      </x:c>
-      <x:c r="H35" s="4" t="n">
-        <x:v>-0.00595619</x:v>
-      </x:c>
-      <x:c r="I35" s="4" t="n">
-        <x:v>0.70160807</x:v>
-      </x:c>
-      <x:c r="J35" s="4" t="n">
-        <x:v>0.01430439</x:v>
       </x:c>
       <x:c r="K35" s="5" t="n">
         <x:v>2700</x:v>
@@ -2575,28 +2715,28 @@
         <x:v>8.75</x:v>
       </x:c>
       <x:c r="C36" s="4" t="n">
+        <x:v>0.07006228</x:v>
+      </x:c>
+      <x:c r="D36" s="4" t="n">
         <x:v>-0.08771841</x:v>
       </x:c>
-      <x:c r="D36" s="4" t="n">
+      <x:c r="E36" s="4" t="n">
+        <x:v>-0.006062809999999999</x:v>
+      </x:c>
+      <x:c r="F36" s="4" t="n">
         <x:v>-0.1425958</x:v>
       </x:c>
-      <x:c r="E36" s="4" t="n">
+      <x:c r="G36" s="4" t="n">
+        <x:v>0.69839586</x:v>
+      </x:c>
+      <x:c r="H36" s="4" t="n">
         <x:v>0.04532014</x:v>
       </x:c>
-      <x:c r="F36" s="4" t="n">
+      <x:c r="I36" s="4" t="n">
+        <x:v>0.01505572</x:v>
+      </x:c>
+      <x:c r="J36" s="4" t="n">
         <x:v>-0.11513861</x:v>
-      </x:c>
-      <x:c r="G36" s="4" t="n">
-        <x:v>0.07006228</x:v>
-      </x:c>
-      <x:c r="H36" s="4" t="n">
-        <x:v>-0.006062809999999999</x:v>
-      </x:c>
-      <x:c r="I36" s="4" t="n">
-        <x:v>0.69839586</x:v>
-      </x:c>
-      <x:c r="J36" s="4" t="n">
-        <x:v>0.01505572</x:v>
       </x:c>
       <x:c r="K36" s="5" t="n">
         <x:v>2700</x:v>
@@ -2631,28 +2771,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="4" t="n">
+        <x:v>0.07019122</x:v>
+      </x:c>
+      <x:c r="D37" s="4" t="n">
         <x:v>-0.08754873999999999</x:v>
       </x:c>
-      <x:c r="D37" s="4" t="n">
+      <x:c r="E37" s="4" t="n">
+        <x:v>-0.00597631</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="n">
         <x:v>-0.14325912000000002</x:v>
       </x:c>
-      <x:c r="E37" s="4" t="n">
+      <x:c r="G37" s="4" t="n">
+        <x:v>0.69716669</x:v>
+      </x:c>
+      <x:c r="H37" s="4" t="n">
         <x:v>0.04225671</x:v>
       </x:c>
-      <x:c r="F37" s="4" t="n">
+      <x:c r="I37" s="4" t="n">
+        <x:v>0.02279277</x:v>
+      </x:c>
+      <x:c r="J37" s="4" t="n">
         <x:v>-0.10706028999999999</x:v>
-      </x:c>
-      <x:c r="G37" s="4" t="n">
-        <x:v>0.07019122</x:v>
-      </x:c>
-      <x:c r="H37" s="4" t="n">
-        <x:v>-0.00597631</x:v>
-      </x:c>
-      <x:c r="I37" s="4" t="n">
-        <x:v>0.69716669</x:v>
-      </x:c>
-      <x:c r="J37" s="4" t="n">
-        <x:v>0.02279277</x:v>
       </x:c>
       <x:c r="K37" s="5" t="n">
         <x:v>2700</x:v>
@@ -2687,28 +2827,28 @@
         <x:v>9.25</x:v>
       </x:c>
       <x:c r="C38" s="4" t="n">
+        <x:v>0.06995066</x:v>
+      </x:c>
+      <x:c r="D38" s="4" t="n">
         <x:v>-0.08764687</x:v>
       </x:c>
-      <x:c r="D38" s="4" t="n">
+      <x:c r="E38" s="4" t="n">
+        <x:v>-0.00553964</x:v>
+      </x:c>
+      <x:c r="F38" s="4" t="n">
         <x:v>-0.14300353</x:v>
       </x:c>
-      <x:c r="E38" s="4" t="n">
+      <x:c r="G38" s="4" t="n">
+        <x:v>0.69509513</x:v>
+      </x:c>
+      <x:c r="H38" s="4" t="n">
         <x:v>0.03792561</x:v>
       </x:c>
-      <x:c r="F38" s="4" t="n">
+      <x:c r="I38" s="4" t="n">
+        <x:v>0.017388840000000003</x:v>
+      </x:c>
+      <x:c r="J38" s="4" t="n">
         <x:v>-0.11350634</x:v>
-      </x:c>
-      <x:c r="G38" s="4" t="n">
-        <x:v>0.06995066</x:v>
-      </x:c>
-      <x:c r="H38" s="4" t="n">
-        <x:v>-0.00553964</x:v>
-      </x:c>
-      <x:c r="I38" s="4" t="n">
-        <x:v>0.69509513</x:v>
-      </x:c>
-      <x:c r="J38" s="4" t="n">
-        <x:v>0.017388840000000003</x:v>
       </x:c>
       <x:c r="K38" s="5" t="n">
         <x:v>2700</x:v>
@@ -2743,28 +2883,28 @@
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="C39" s="4" t="n">
+        <x:v>0.06995791999999999</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="n">
         <x:v>-0.08725006</x:v>
       </x:c>
-      <x:c r="D39" s="4" t="n">
+      <x:c r="E39" s="4" t="n">
+        <x:v>-0.0044663</x:v>
+      </x:c>
+      <x:c r="F39" s="4" t="n">
         <x:v>-0.14225091</x:v>
       </x:c>
-      <x:c r="E39" s="4" t="n">
+      <x:c r="G39" s="4" t="n">
+        <x:v>0.6947220900000001</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="n">
         <x:v>0.0357702</x:v>
       </x:c>
-      <x:c r="F39" s="4" t="n">
+      <x:c r="I39" s="4" t="n">
+        <x:v>0.01737249</x:v>
+      </x:c>
+      <x:c r="J39" s="4" t="n">
         <x:v>-0.11531788000000001</x:v>
-      </x:c>
-      <x:c r="G39" s="4" t="n">
-        <x:v>0.06995791999999999</x:v>
-      </x:c>
-      <x:c r="H39" s="4" t="n">
-        <x:v>-0.0044663</x:v>
-      </x:c>
-      <x:c r="I39" s="4" t="n">
-        <x:v>0.6947220900000001</x:v>
-      </x:c>
-      <x:c r="J39" s="4" t="n">
-        <x:v>0.01737249</x:v>
       </x:c>
       <x:c r="K39" s="5" t="n">
         <x:v>2700</x:v>
@@ -2799,28 +2939,28 @@
         <x:v>9.75</x:v>
       </x:c>
       <x:c r="C40" s="4" t="n">
+        <x:v>0.06985364</x:v>
+      </x:c>
+      <x:c r="D40" s="4" t="n">
         <x:v>-0.08703288</x:v>
       </x:c>
-      <x:c r="D40" s="4" t="n">
+      <x:c r="E40" s="4" t="n">
+        <x:v>-0.005000360000000001</x:v>
+      </x:c>
+      <x:c r="F40" s="4" t="n">
         <x:v>-0.14332185</x:v>
       </x:c>
-      <x:c r="E40" s="4" t="n">
+      <x:c r="G40" s="4" t="n">
+        <x:v>0.69425637</x:v>
+      </x:c>
+      <x:c r="H40" s="4" t="n">
         <x:v>0.034069630000000004</x:v>
       </x:c>
-      <x:c r="F40" s="4" t="n">
+      <x:c r="I40" s="4" t="n">
+        <x:v>0.018463419999999998</x:v>
+      </x:c>
+      <x:c r="J40" s="4" t="n">
         <x:v>-0.11525044</x:v>
-      </x:c>
-      <x:c r="G40" s="4" t="n">
-        <x:v>0.06985364</x:v>
-      </x:c>
-      <x:c r="H40" s="4" t="n">
-        <x:v>-0.005000360000000001</x:v>
-      </x:c>
-      <x:c r="I40" s="4" t="n">
-        <x:v>0.69425637</x:v>
-      </x:c>
-      <x:c r="J40" s="4" t="n">
-        <x:v>0.018463419999999998</x:v>
       </x:c>
       <x:c r="K40" s="5" t="n">
         <x:v>2700</x:v>
@@ -2855,28 +2995,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C41" s="4" t="n">
+        <x:v>0.06988264</x:v>
+      </x:c>
+      <x:c r="D41" s="4" t="n">
         <x:v>-0.08705237</x:v>
       </x:c>
-      <x:c r="D41" s="4" t="n">
+      <x:c r="E41" s="4" t="n">
+        <x:v>-0.00515605</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="n">
         <x:v>-0.14394679</x:v>
       </x:c>
-      <x:c r="E41" s="4" t="n">
+      <x:c r="G41" s="4" t="n">
+        <x:v>0.6941789</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="n">
         <x:v>0.03233765</x:v>
       </x:c>
-      <x:c r="F41" s="4" t="n">
+      <x:c r="I41" s="4" t="n">
+        <x:v>0.02430999</x:v>
+      </x:c>
+      <x:c r="J41" s="4" t="n">
         <x:v>-0.10899497999999999</x:v>
-      </x:c>
-      <x:c r="G41" s="4" t="n">
-        <x:v>0.06988264</x:v>
-      </x:c>
-      <x:c r="H41" s="4" t="n">
-        <x:v>-0.00515605</x:v>
-      </x:c>
-      <x:c r="I41" s="4" t="n">
-        <x:v>0.6941789</x:v>
-      </x:c>
-      <x:c r="J41" s="4" t="n">
-        <x:v>0.02430999</x:v>
       </x:c>
       <x:c r="K41" s="5" t="n">
         <x:v>2700</x:v>
@@ -2905,9 +3045,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11d41c15fec14012"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65fccb1f72b54f2f"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd1ea359d4da4430"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf391e7f9da684b56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use time-weighted annual returns in forward exports
</commit_message>
<xml_diff>
--- a/analysis/forward_beat_curves_wide.xlsx
+++ b/analysis/forward_beat_curves_wide.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Beats Wide" sheetId="1" r:id="Ra5c9db24553948d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward Beats Wide" sheetId="1" r:id="Rc1d2c6f5dc124dbd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,7 +497,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc6dc6198b524996"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85efa81628414f1c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -867,19 +867,19 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="C3" s="4" t="n">
-        <x:v>0.39233845</x:v>
+        <x:v>0.38118220999999997</x:v>
       </x:c>
       <x:c r="D3" s="4" t="n">
         <x:v>0.24759328</x:v>
       </x:c>
       <x:c r="E3" s="4" t="n">
-        <x:v>0.05057315</x:v>
+        <x:v>0.0500009</x:v>
       </x:c>
       <x:c r="F3" s="4" t="n">
         <x:v>-0.07124741</x:v>
       </x:c>
       <x:c r="G3" s="4" t="n">
-        <x:v>1.7213936699999999</x:v>
+        <x:v>1.5720725</x:v>
       </x:c>
       <x:c r="H3" s="4" t="n">
         <x:v>1.44225412</x:v>
@@ -923,25 +923,25 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="C4" s="4" t="n">
-        <x:v>0.24742139999999999</x:v>
+        <x:v>0.23069671</x:v>
       </x:c>
       <x:c r="D4" s="4" t="n">
         <x:v>0.10602118</x:v>
       </x:c>
       <x:c r="E4" s="4" t="n">
-        <x:v>-0.0084732</x:v>
+        <x:v>-0.00978715</x:v>
       </x:c>
       <x:c r="F4" s="4" t="n">
         <x:v>-0.12657378</x:v>
       </x:c>
       <x:c r="G4" s="4" t="n">
-        <x:v>1.1123960099999999</x:v>
+        <x:v>0.89143337</x:v>
       </x:c>
       <x:c r="H4" s="4" t="n">
         <x:v>0.7858886599999999</x:v>
       </x:c>
       <x:c r="I4" s="4" t="n">
-        <x:v>0.06271391999999999</x:v>
+        <x:v>0.06245528</x:v>
       </x:c>
       <x:c r="J4" s="4" t="n">
         <x:v>-0.03363994</x:v>
@@ -979,25 +979,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
-        <x:v>0.17331331</x:v>
+        <x:v>0.1529898</x:v>
       </x:c>
       <x:c r="D5" s="4" t="n">
         <x:v>0.03237439</x:v>
       </x:c>
       <x:c r="E5" s="4" t="n">
-        <x:v>-0.025765660000000003</x:v>
+        <x:v>-0.02741681</x:v>
       </x:c>
       <x:c r="F5" s="4" t="n">
         <x:v>-0.13809864</x:v>
       </x:c>
       <x:c r="G5" s="4" t="n">
-        <x:v>0.88268027</x:v>
+        <x:v>0.62289695</x:v>
       </x:c>
       <x:c r="H5" s="4" t="n">
         <x:v>0.5293873099999999</x:v>
       </x:c>
       <x:c r="I5" s="4" t="n">
-        <x:v>0.02088956</x:v>
+        <x:v>0.019454469999999998</x:v>
       </x:c>
       <x:c r="J5" s="4" t="n">
         <x:v>-0.06953677</x:v>
@@ -1035,25 +1035,25 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
-        <x:v>0.14220753</x:v>
+        <x:v>0.11798879</x:v>
       </x:c>
       <x:c r="D6" s="4" t="n">
         <x:v>0.00002065</x:v>
       </x:c>
       <x:c r="E6" s="4" t="n">
-        <x:v>-0.03905462</x:v>
+        <x:v>-0.04103339</x:v>
       </x:c>
       <x:c r="F6" s="4" t="n">
         <x:v>-0.15179735</x:v>
       </x:c>
       <x:c r="G6" s="4" t="n">
-        <x:v>0.8366828</x:v>
+        <x:v>0.52018017</x:v>
       </x:c>
       <x:c r="H6" s="4" t="n">
         <x:v>0.43496505999999996</x:v>
       </x:c>
       <x:c r="I6" s="4" t="n">
-        <x:v>0.01031148</x:v>
+        <x:v>0.0081421</x:v>
       </x:c>
       <x:c r="J6" s="4" t="n">
         <x:v>-0.08539844</x:v>
@@ -1091,25 +1091,25 @@
         <x:v>1.5</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
-        <x:v>0.12556831000000002</x:v>
+        <x:v>0.09919385</x:v>
       </x:c>
       <x:c r="D7" s="4" t="n">
         <x:v>-0.019649859999999998</x:v>
       </x:c>
       <x:c r="E7" s="4" t="n">
-        <x:v>-0.04314972</x:v>
+        <x:v>-0.04563599</x:v>
       </x:c>
       <x:c r="F7" s="4" t="n">
         <x:v>-0.15583248</x:v>
       </x:c>
       <x:c r="G7" s="4" t="n">
-        <x:v>0.7901467200000001</x:v>
+        <x:v>0.43358129</x:v>
       </x:c>
       <x:c r="H7" s="4" t="n">
         <x:v>0.3421975</x:v>
       </x:c>
       <x:c r="I7" s="4" t="n">
-        <x:v>0.01340144</x:v>
+        <x:v>0.00952176</x:v>
       </x:c>
       <x:c r="J7" s="4" t="n">
         <x:v>-0.07935047</x:v>
@@ -1147,25 +1147,25 @@
         <x:v>1.75</x:v>
       </x:c>
       <x:c r="C8" s="4" t="n">
-        <x:v>0.11094817000000001</x:v>
+        <x:v>0.08291791</x:v>
       </x:c>
       <x:c r="D8" s="4" t="n">
         <x:v>-0.03743142</x:v>
       </x:c>
       <x:c r="E8" s="4" t="n">
-        <x:v>-0.043118210000000004</x:v>
+        <x:v>-0.046157250000000004</x:v>
       </x:c>
       <x:c r="F8" s="4" t="n">
         <x:v>-0.15784511</x:v>
       </x:c>
       <x:c r="G8" s="4" t="n">
-        <x:v>0.77526989</x:v>
+        <x:v>0.38998500999999997</x:v>
       </x:c>
       <x:c r="H8" s="4" t="n">
         <x:v>0.30150953999999996</x:v>
       </x:c>
       <x:c r="I8" s="4" t="n">
-        <x:v>-0.0031502200000000005</x:v>
+        <x:v>-0.00872581</x:v>
       </x:c>
       <x:c r="J8" s="4" t="n">
         <x:v>-0.10121532999999999</x:v>
@@ -1203,25 +1203,25 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="4" t="n">
-        <x:v>0.10255887</x:v>
+        <x:v>0.07342061</x:v>
       </x:c>
       <x:c r="D9" s="4" t="n">
         <x:v>-0.047021610000000005</x:v>
       </x:c>
       <x:c r="E9" s="4" t="n">
-        <x:v>-0.04105271</x:v>
+        <x:v>-0.04452318</x:v>
       </x:c>
       <x:c r="F9" s="4" t="n">
         <x:v>-0.15668238</x:v>
       </x:c>
       <x:c r="G9" s="4" t="n">
-        <x:v>0.78729079</x:v>
+        <x:v>0.38189366</x:v>
       </x:c>
       <x:c r="H9" s="4" t="n">
         <x:v>0.2870739</x:v>
       </x:c>
       <x:c r="I9" s="4" t="n">
-        <x:v>0.0072936</x:v>
+        <x:v>0.00083387</x:v>
       </x:c>
       <x:c r="J9" s="4" t="n">
         <x:v>-0.0897294</x:v>
@@ -1259,25 +1259,25 @@
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="C10" s="4" t="n">
-        <x:v>0.09505528999999999</x:v>
+        <x:v>0.06485229</x:v>
       </x:c>
       <x:c r="D10" s="4" t="n">
         <x:v>-0.05614853</x:v>
       </x:c>
       <x:c r="E10" s="4" t="n">
-        <x:v>-0.04450799</x:v>
+        <x:v>-0.04856356</x:v>
       </x:c>
       <x:c r="F10" s="4" t="n">
         <x:v>-0.16062328999999997</x:v>
       </x:c>
       <x:c r="G10" s="4" t="n">
-        <x:v>0.76466207</x:v>
+        <x:v>0.3408206</x:v>
       </x:c>
       <x:c r="H10" s="4" t="n">
         <x:v>0.24808847</x:v>
       </x:c>
       <x:c r="I10" s="4" t="n">
-        <x:v>0.00750408</x:v>
+        <x:v>0.00028314</x:v>
       </x:c>
       <x:c r="J10" s="4" t="n">
         <x:v>-0.08441209000000001</x:v>
@@ -1315,25 +1315,25 @@
         <x:v>2.5</x:v>
       </x:c>
       <x:c r="C11" s="4" t="n">
-        <x:v>0.09002432</x:v>
+        <x:v>0.05903213</x:v>
       </x:c>
       <x:c r="D11" s="4" t="n">
         <x:v>-0.06250963999999999</x:v>
       </x:c>
       <x:c r="E11" s="4" t="n">
-        <x:v>-0.04176406</x:v>
+        <x:v>-0.04618363</x:v>
       </x:c>
       <x:c r="F11" s="4" t="n">
         <x:v>-0.15901998</x:v>
       </x:c>
       <x:c r="G11" s="4" t="n">
-        <x:v>0.77425814</x:v>
+        <x:v>0.33828068</x:v>
       </x:c>
       <x:c r="H11" s="4" t="n">
         <x:v>0.24771844999999998</x:v>
       </x:c>
       <x:c r="I11" s="4" t="n">
-        <x:v>0.01118937</x:v>
+        <x:v>0.00320646</x:v>
       </x:c>
       <x:c r="J11" s="4" t="n">
         <x:v>-0.08032844</x:v>
@@ -1371,25 +1371,25 @@
         <x:v>2.75</x:v>
       </x:c>
       <x:c r="C12" s="4" t="n">
-        <x:v>0.09202362000000001</x:v>
+        <x:v>0.060910469999999994</x:v>
       </x:c>
       <x:c r="D12" s="4" t="n">
         <x:v>-0.06244242</x:v>
       </x:c>
       <x:c r="E12" s="4" t="n">
-        <x:v>-0.037324989999999995</x:v>
+        <x:v>-0.042021670000000004</x:v>
       </x:c>
       <x:c r="F12" s="4" t="n">
         <x:v>-0.15588558</x:v>
       </x:c>
       <x:c r="G12" s="4" t="n">
-        <x:v>0.77355458</x:v>
+        <x:v>0.32654451</x:v>
       </x:c>
       <x:c r="H12" s="4" t="n">
         <x:v>0.23519313</x:v>
       </x:c>
       <x:c r="I12" s="4" t="n">
-        <x:v>0.02009764</x:v>
+        <x:v>0.01126969</x:v>
       </x:c>
       <x:c r="J12" s="4" t="n">
         <x:v>-0.06969739</x:v>
@@ -1427,25 +1427,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="4" t="n">
-        <x:v>0.08932176</x:v>
+        <x:v>0.05796689</x:v>
       </x:c>
       <x:c r="D13" s="4" t="n">
         <x:v>-0.06673396000000001</x:v>
       </x:c>
       <x:c r="E13" s="4" t="n">
-        <x:v>-0.03847424</x:v>
+        <x:v>-0.04366314</x:v>
       </x:c>
       <x:c r="F13" s="4" t="n">
         <x:v>-0.15814809</x:v>
       </x:c>
       <x:c r="G13" s="4" t="n">
-        <x:v>0.75996892</x:v>
+        <x:v>0.30185975</x:v>
       </x:c>
       <x:c r="H13" s="4" t="n">
         <x:v>0.21080369000000002</x:v>
       </x:c>
       <x:c r="I13" s="4" t="n">
-        <x:v>0.032826970000000004</x:v>
+        <x:v>0.02379598</x:v>
       </x:c>
       <x:c r="J13" s="4" t="n">
         <x:v>-0.05835143</x:v>
@@ -1483,25 +1483,25 @@
         <x:v>3.25</x:v>
       </x:c>
       <x:c r="C14" s="4" t="n">
-        <x:v>0.08613728999999999</x:v>
+        <x:v>0.05444923</x:v>
       </x:c>
       <x:c r="D14" s="4" t="n">
         <x:v>-0.07138751</x:v>
       </x:c>
       <x:c r="E14" s="4" t="n">
-        <x:v>-0.03398754</x:v>
+        <x:v>-0.0394565</x:v>
       </x:c>
       <x:c r="F14" s="4" t="n">
         <x:v>-0.15493949</x:v>
       </x:c>
       <x:c r="G14" s="4" t="n">
-        <x:v>0.7610820300000001</x:v>
+        <x:v>0.29506779</x:v>
       </x:c>
       <x:c r="H14" s="4" t="n">
         <x:v>0.20091024999999998</x:v>
       </x:c>
       <x:c r="I14" s="4" t="n">
-        <x:v>0.0257943</x:v>
+        <x:v>0.0157357</x:v>
       </x:c>
       <x:c r="J14" s="4" t="n">
         <x:v>-0.06947901</x:v>
@@ -1539,25 +1539,25 @@
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="C15" s="4" t="n">
-        <x:v>0.08456089</x:v>
+        <x:v>0.052884650000000005</x:v>
       </x:c>
       <x:c r="D15" s="4" t="n">
         <x:v>-0.07296469</x:v>
       </x:c>
       <x:c r="E15" s="4" t="n">
-        <x:v>-0.032100529999999995</x:v>
+        <x:v>-0.03786627</x:v>
       </x:c>
       <x:c r="F15" s="4" t="n">
         <x:v>-0.15410417</x:v>
       </x:c>
       <x:c r="G15" s="4" t="n">
-        <x:v>0.7530800999999999</x:v>
+        <x:v>0.27885508000000003</x:v>
       </x:c>
       <x:c r="H15" s="4" t="n">
         <x:v>0.18524174999999998</x:v>
       </x:c>
       <x:c r="I15" s="4" t="n">
-        <x:v>0.023804759999999998</x:v>
+        <x:v>0.013165020000000001</x:v>
       </x:c>
       <x:c r="J15" s="4" t="n">
         <x:v>-0.07203282</x:v>
@@ -1595,25 +1595,25 @@
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="C16" s="4" t="n">
-        <x:v>0.08314926</x:v>
+        <x:v>0.05167694</x:v>
       </x:c>
       <x:c r="D16" s="4" t="n">
         <x:v>-0.07487475</x:v>
       </x:c>
       <x:c r="E16" s="4" t="n">
-        <x:v>-0.03220619</x:v>
+        <x:v>-0.038357869999999995</x:v>
       </x:c>
       <x:c r="F16" s="4" t="n">
         <x:v>-0.15546027</x:v>
       </x:c>
       <x:c r="G16" s="4" t="n">
-        <x:v>0.73816616</x:v>
+        <x:v>0.25538304</x:v>
       </x:c>
       <x:c r="H16" s="4" t="n">
         <x:v>0.16269943</x:v>
       </x:c>
       <x:c r="I16" s="4" t="n">
-        <x:v>-0.0046911900000000005</x:v>
+        <x:v>-0.01744938</x:v>
       </x:c>
       <x:c r="J16" s="4" t="n">
         <x:v>-0.10291204000000001</x:v>
@@ -1651,25 +1651,25 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C17" s="4" t="n">
-        <x:v>0.08002729</x:v>
+        <x:v>0.04870494</x:v>
       </x:c>
       <x:c r="D17" s="4" t="n">
         <x:v>-0.07866987</x:v>
       </x:c>
       <x:c r="E17" s="4" t="n">
-        <x:v>-0.02629399</x:v>
+        <x:v>-0.03246901</x:v>
       </x:c>
       <x:c r="F17" s="4" t="n">
         <x:v>-0.15016864</x:v>
       </x:c>
       <x:c r="G17" s="4" t="n">
-        <x:v>0.73486666</x:v>
+        <x:v>0.24601140000000002</x:v>
       </x:c>
       <x:c r="H17" s="4" t="n">
         <x:v>0.14919665000000001</x:v>
       </x:c>
       <x:c r="I17" s="4" t="n">
-        <x:v>0.01501994</x:v>
+        <x:v>0.0019126000000000002</x:v>
       </x:c>
       <x:c r="J17" s="4" t="n">
         <x:v>-0.08682121999999999</x:v>
@@ -1707,25 +1707,25 @@
         <x:v>4.25</x:v>
       </x:c>
       <x:c r="C18" s="4" t="n">
-        <x:v>0.07890989</x:v>
+        <x:v>0.04797001</x:v>
       </x:c>
       <x:c r="D18" s="4" t="n">
         <x:v>-0.0795706</x:v>
       </x:c>
       <x:c r="E18" s="4" t="n">
-        <x:v>-0.02630046</x:v>
+        <x:v>-0.03297468</x:v>
       </x:c>
       <x:c r="F18" s="4" t="n">
         <x:v>-0.15145261</x:v>
       </x:c>
       <x:c r="G18" s="4" t="n">
-        <x:v>0.71473337</x:v>
+        <x:v>0.21806525000000002</x:v>
       </x:c>
       <x:c r="H18" s="4" t="n">
         <x:v>0.12224317</x:v>
       </x:c>
       <x:c r="I18" s="4" t="n">
-        <x:v>-0.00227935</x:v>
+        <x:v>-0.0168384</x:v>
       </x:c>
       <x:c r="J18" s="4" t="n">
         <x:v>-0.11122488000000001</x:v>
@@ -1763,25 +1763,25 @@
         <x:v>4.5</x:v>
       </x:c>
       <x:c r="C19" s="4" t="n">
-        <x:v>0.07733747</x:v>
+        <x:v>0.04677849</x:v>
       </x:c>
       <x:c r="D19" s="4" t="n">
         <x:v>-0.08127632</x:v>
       </x:c>
       <x:c r="E19" s="4" t="n">
-        <x:v>-0.024729619999999997</x:v>
+        <x:v>-0.0317633</x:v>
       </x:c>
       <x:c r="F19" s="4" t="n">
         <x:v>-0.15081706</x:v>
       </x:c>
       <x:c r="G19" s="4" t="n">
-        <x:v>0.70834075</x:v>
+        <x:v>0.20629269</x:v>
       </x:c>
       <x:c r="H19" s="4" t="n">
         <x:v>0.1099639</x:v>
       </x:c>
       <x:c r="I19" s="4" t="n">
-        <x:v>-0.0019506100000000002</x:v>
+        <x:v>-0.01721581</x:v>
       </x:c>
       <x:c r="J19" s="4" t="n">
         <x:v>-0.1137833</x:v>
@@ -1819,25 +1819,25 @@
         <x:v>4.75</x:v>
       </x:c>
       <x:c r="C20" s="4" t="n">
-        <x:v>0.07675477</x:v>
+        <x:v>0.046780249999999995</x:v>
       </x:c>
       <x:c r="D20" s="4" t="n">
         <x:v>-0.08175044</x:v>
       </x:c>
       <x:c r="E20" s="4" t="n">
-        <x:v>-0.02104819</x:v>
+        <x:v>-0.02810962</x:v>
       </x:c>
       <x:c r="F20" s="4" t="n">
         <x:v>-0.14733241</x:v>
       </x:c>
       <x:c r="G20" s="4" t="n">
-        <x:v>0.71559037</x:v>
+        <x:v>0.21110872</x:v>
       </x:c>
       <x:c r="H20" s="4" t="n">
         <x:v>0.11277879</x:v>
       </x:c>
       <x:c r="I20" s="4" t="n">
-        <x:v>0.0114879</x:v>
+        <x:v>-0.0034173999999999997</x:v>
       </x:c>
       <x:c r="J20" s="4" t="n">
         <x:v>-0.09378943</x:v>
@@ -1875,25 +1875,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="4" t="n">
-        <x:v>0.0758809</x:v>
+        <x:v>0.046392569999999994</x:v>
       </x:c>
       <x:c r="D21" s="4" t="n">
         <x:v>-0.08194342</x:v>
       </x:c>
       <x:c r="E21" s="4" t="n">
-        <x:v>-0.01856386</x:v>
+        <x:v>-0.02569775</x:v>
       </x:c>
       <x:c r="F21" s="4" t="n">
         <x:v>-0.1447298</x:v>
       </x:c>
       <x:c r="G21" s="4" t="n">
-        <x:v>0.71062455</x:v>
+        <x:v>0.20167922000000002</x:v>
       </x:c>
       <x:c r="H21" s="4" t="n">
         <x:v>0.10344272</x:v>
       </x:c>
       <x:c r="I21" s="4" t="n">
-        <x:v>0.00246159</x:v>
+        <x:v>-0.0130787</x:v>
       </x:c>
       <x:c r="J21" s="4" t="n">
         <x:v>-0.10493866</x:v>
@@ -1931,25 +1931,25 @@
         <x:v>5.25</x:v>
       </x:c>
       <x:c r="C22" s="4" t="n">
-        <x:v>0.07514735</x:v>
+        <x:v>0.046120799999999997</x:v>
       </x:c>
       <x:c r="D22" s="4" t="n">
         <x:v>-0.08276863000000001</x:v>
       </x:c>
       <x:c r="E22" s="4" t="n">
-        <x:v>-0.01741189</x:v>
+        <x:v>-0.024731640000000003</x:v>
       </x:c>
       <x:c r="F22" s="4" t="n">
         <x:v>-0.14502652</x:v>
       </x:c>
       <x:c r="G22" s="4" t="n">
-        <x:v>0.7134843700000001</x:v>
+        <x:v>0.20191166</x:v>
       </x:c>
       <x:c r="H22" s="4" t="n">
         <x:v>0.10237738</x:v>
       </x:c>
       <x:c r="I22" s="4" t="n">
-        <x:v>0.00423328</x:v>
+        <x:v>-0.01199125</x:v>
       </x:c>
       <x:c r="J22" s="4" t="n">
         <x:v>-0.10697424</x:v>
@@ -1987,25 +1987,25 @@
         <x:v>5.5</x:v>
       </x:c>
       <x:c r="C23" s="4" t="n">
-        <x:v>0.07401562</x:v>
+        <x:v>0.04521025</x:v>
       </x:c>
       <x:c r="D23" s="4" t="n">
         <x:v>-0.08444378000000001</x:v>
       </x:c>
       <x:c r="E23" s="4" t="n">
-        <x:v>-0.016525579999999998</x:v>
+        <x:v>-0.023998330000000002</x:v>
       </x:c>
       <x:c r="F23" s="4" t="n">
         <x:v>-0.14541458000000002</x:v>
       </x:c>
       <x:c r="G23" s="4" t="n">
-        <x:v>0.71274644</x:v>
+        <x:v>0.19800308</x:v>
       </x:c>
       <x:c r="H23" s="4" t="n">
         <x:v>0.09812398</x:v>
       </x:c>
       <x:c r="I23" s="4" t="n">
-        <x:v>0.00000193</x:v>
+        <x:v>-0.01676229</x:v>
       </x:c>
       <x:c r="J23" s="4" t="n">
         <x:v>-0.11284015</x:v>
@@ -2043,25 +2043,25 @@
         <x:v>5.75</x:v>
       </x:c>
       <x:c r="C24" s="4" t="n">
-        <x:v>0.07311567000000001</x:v>
+        <x:v>0.04455558</x:v>
       </x:c>
       <x:c r="D24" s="4" t="n">
         <x:v>-0.08521266000000001</x:v>
       </x:c>
       <x:c r="E24" s="4" t="n">
-        <x:v>-0.015606580000000002</x:v>
+        <x:v>-0.02320891</x:v>
       </x:c>
       <x:c r="F24" s="4" t="n">
         <x:v>-0.14551841</x:v>
       </x:c>
       <x:c r="G24" s="4" t="n">
-        <x:v>0.71128163</x:v>
+        <x:v>0.19364667000000002</x:v>
       </x:c>
       <x:c r="H24" s="4" t="n">
         <x:v>0.09152996</x:v>
       </x:c>
       <x:c r="I24" s="4" t="n">
-        <x:v>0.00748991</x:v>
+        <x:v>-0.0090039</x:v>
       </x:c>
       <x:c r="J24" s="4" t="n">
         <x:v>-0.10432454999999999</x:v>
@@ -2099,25 +2099,25 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C25" s="4" t="n">
-        <x:v>0.07292462000000001</x:v>
+        <x:v>0.04477558</x:v>
       </x:c>
       <x:c r="D25" s="4" t="n">
         <x:v>-0.08517493999999999</x:v>
       </x:c>
       <x:c r="E25" s="4" t="n">
-        <x:v>-0.015038339999999999</x:v>
+        <x:v>-0.02281281</x:v>
       </x:c>
       <x:c r="F25" s="4" t="n">
         <x:v>-0.145875</x:v>
       </x:c>
       <x:c r="G25" s="4" t="n">
-        <x:v>0.7140234599999999</x:v>
+        <x:v>0.1946548</x:v>
       </x:c>
       <x:c r="H25" s="4" t="n">
         <x:v>0.09248946999999999</x:v>
       </x:c>
       <x:c r="I25" s="4" t="n">
-        <x:v>-0.00367682</x:v>
+        <x:v>-0.021601699999999998</x:v>
       </x:c>
       <x:c r="J25" s="4" t="n">
         <x:v>-0.11794807</x:v>
@@ -2155,25 +2155,25 @@
         <x:v>6.25</x:v>
       </x:c>
       <x:c r="C26" s="4" t="n">
-        <x:v>0.07242833</x:v>
+        <x:v>0.04457363</x:v>
       </x:c>
       <x:c r="D26" s="4" t="n">
         <x:v>-0.08581214</x:v>
       </x:c>
       <x:c r="E26" s="4" t="n">
-        <x:v>-0.013203769999999998</x:v>
+        <x:v>-0.020923709999999998</x:v>
       </x:c>
       <x:c r="F26" s="4" t="n">
         <x:v>-0.14449087</x:v>
       </x:c>
       <x:c r="G26" s="4" t="n">
-        <x:v>0.71447977</x:v>
+        <x:v>0.19301390000000002</x:v>
       </x:c>
       <x:c r="H26" s="4" t="n">
         <x:v>0.09077088</x:v>
       </x:c>
       <x:c r="I26" s="4" t="n">
-        <x:v>0.00370828</x:v>
+        <x:v>-0.01433485</x:v>
       </x:c>
       <x:c r="J26" s="4" t="n">
         <x:v>-0.11050867</x:v>
@@ -2211,25 +2211,25 @@
         <x:v>6.5</x:v>
       </x:c>
       <x:c r="C27" s="4" t="n">
-        <x:v>0.07244373</x:v>
+        <x:v>0.04501243</x:v>
       </x:c>
       <x:c r="D27" s="4" t="n">
         <x:v>-0.08565292</x:v>
       </x:c>
       <x:c r="E27" s="4" t="n">
-        <x:v>-0.01156242</x:v>
+        <x:v>-0.01922134</x:v>
       </x:c>
       <x:c r="F27" s="4" t="n">
         <x:v>-0.14310118</x:v>
       </x:c>
       <x:c r="G27" s="4" t="n">
-        <x:v>0.71410273</x:v>
+        <x:v>0.19048948</x:v>
       </x:c>
       <x:c r="H27" s="4" t="n">
         <x:v>0.08589905999999999</x:v>
       </x:c>
       <x:c r="I27" s="4" t="n">
-        <x:v>-0.0025236300000000002</x:v>
+        <x:v>-0.021013860000000002</x:v>
       </x:c>
       <x:c r="J27" s="4" t="n">
         <x:v>-0.11914403999999999</x:v>
@@ -2267,25 +2267,25 @@
         <x:v>6.75</x:v>
       </x:c>
       <x:c r="C28" s="4" t="n">
-        <x:v>0.07197154</x:v>
+        <x:v>0.04481364</x:v>
       </x:c>
       <x:c r="D28" s="4" t="n">
         <x:v>-0.08625392</x:v>
       </x:c>
       <x:c r="E28" s="4" t="n">
-        <x:v>-0.01052451</x:v>
+        <x:v>-0.01817877</x:v>
       </x:c>
       <x:c r="F28" s="4" t="n">
         <x:v>-0.14275758</x:v>
       </x:c>
       <x:c r="G28" s="4" t="n">
-        <x:v>0.71277247</x:v>
+        <x:v>0.18689737</x:v>
       </x:c>
       <x:c r="H28" s="4" t="n">
         <x:v>0.08106661000000001</x:v>
       </x:c>
       <x:c r="I28" s="4" t="n">
-        <x:v>0.00473786</x:v>
+        <x:v>-0.01390664</x:v>
       </x:c>
       <x:c r="J28" s="4" t="n">
         <x:v>-0.11286602999999999</x:v>
@@ -2323,25 +2323,25 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C29" s="4" t="n">
-        <x:v>0.07099008000000001</x:v>
+        <x:v>0.04393601999999999</x:v>
       </x:c>
       <x:c r="D29" s="4" t="n">
         <x:v>-0.08724453</x:v>
       </x:c>
       <x:c r="E29" s="4" t="n">
-        <x:v>-0.01057723</x:v>
+        <x:v>-0.018502559999999998</x:v>
       </x:c>
       <x:c r="F29" s="4" t="n">
         <x:v>-0.14385314</x:v>
       </x:c>
       <x:c r="G29" s="4" t="n">
-        <x:v>0.71119622</x:v>
+        <x:v>0.1829887</x:v>
       </x:c>
       <x:c r="H29" s="4" t="n">
         <x:v>0.07626068</x:v>
       </x:c>
       <x:c r="I29" s="4" t="n">
-        <x:v>-0.00876789</x:v>
+        <x:v>-0.03023102</x:v>
       </x:c>
       <x:c r="J29" s="4" t="n">
         <x:v>-0.133162</x:v>
@@ -2379,25 +2379,25 @@
         <x:v>7.25</x:v>
       </x:c>
       <x:c r="C30" s="4" t="n">
-        <x:v>0.07098623</x:v>
+        <x:v>0.04432124</x:v>
       </x:c>
       <x:c r="D30" s="4" t="n">
         <x:v>-0.08675118</x:v>
       </x:c>
       <x:c r="E30" s="4" t="n">
-        <x:v>-0.00840723</x:v>
+        <x:v>-0.01599435</x:v>
       </x:c>
       <x:c r="F30" s="4" t="n">
         <x:v>-0.14204597</x:v>
       </x:c>
       <x:c r="G30" s="4" t="n">
-        <x:v>0.70595303</x:v>
+        <x:v>0.17443730999999998</x:v>
       </x:c>
       <x:c r="H30" s="4" t="n">
         <x:v>0.07025065999999999</x:v>
       </x:c>
       <x:c r="I30" s="4" t="n">
-        <x:v>0.0120945</x:v>
+        <x:v>-0.00695368</x:v>
       </x:c>
       <x:c r="J30" s="4" t="n">
         <x:v>-0.10940025</x:v>
@@ -2435,25 +2435,25 @@
         <x:v>7.5</x:v>
       </x:c>
       <x:c r="C31" s="4" t="n">
-        <x:v>0.07061128</x:v>
+        <x:v>0.04416962</x:v>
       </x:c>
       <x:c r="D31" s="4" t="n">
         <x:v>-0.08724768</x:v>
       </x:c>
       <x:c r="E31" s="4" t="n">
-        <x:v>-0.00827957</x:v>
+        <x:v>-0.01603565</x:v>
       </x:c>
       <x:c r="F31" s="4" t="n">
         <x:v>-0.14238759</x:v>
       </x:c>
       <x:c r="G31" s="4" t="n">
-        <x:v>0.7043785300000001</x:v>
+        <x:v>0.17064354999999998</x:v>
       </x:c>
       <x:c r="H31" s="4" t="n">
         <x:v>0.06497098</x:v>
       </x:c>
       <x:c r="I31" s="4" t="n">
-        <x:v>0.00368604</x:v>
+        <x:v>-0.017107090000000002</x:v>
       </x:c>
       <x:c r="J31" s="4" t="n">
         <x:v>-0.11961812</x:v>
@@ -2491,25 +2491,25 @@
         <x:v>7.75</x:v>
       </x:c>
       <x:c r="C32" s="4" t="n">
-        <x:v>0.06992869</x:v>
+        <x:v>0.04357692</x:v>
       </x:c>
       <x:c r="D32" s="4" t="n">
         <x:v>-0.08771672999999999</x:v>
       </x:c>
       <x:c r="E32" s="4" t="n">
-        <x:v>-0.00995782</x:v>
+        <x:v>-0.01842446</x:v>
       </x:c>
       <x:c r="F32" s="4" t="n">
         <x:v>-0.14565065</x:v>
       </x:c>
       <x:c r="G32" s="4" t="n">
-        <x:v>0.7050791099999999</x:v>
+        <x:v>0.16984801000000002</x:v>
       </x:c>
       <x:c r="H32" s="4" t="n">
         <x:v>0.06390123</x:v>
       </x:c>
       <x:c r="I32" s="4" t="n">
-        <x:v>0.00901543</x:v>
+        <x:v>-0.01089751</x:v>
       </x:c>
       <x:c r="J32" s="4" t="n">
         <x:v>-0.11825642</x:v>
@@ -2547,25 +2547,25 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="4" t="n">
-        <x:v>0.07037093</x:v>
+        <x:v>0.04451598</x:v>
       </x:c>
       <x:c r="D33" s="4" t="n">
         <x:v>-0.08746663</x:v>
       </x:c>
       <x:c r="E33" s="4" t="n">
-        <x:v>-0.00870937</x:v>
+        <x:v>-0.01704149</x:v>
       </x:c>
       <x:c r="F33" s="4" t="n">
         <x:v>-0.14435053</x:v>
       </x:c>
       <x:c r="G33" s="4" t="n">
-        <x:v>0.7061083100000001</x:v>
+        <x:v>0.16951298999999997</x:v>
       </x:c>
       <x:c r="H33" s="4" t="n">
         <x:v>0.062249679999999995</x:v>
       </x:c>
       <x:c r="I33" s="4" t="n">
-        <x:v>0.007530909999999999</x:v>
+        <x:v>-0.01311986</x:v>
       </x:c>
       <x:c r="J33" s="4" t="n">
         <x:v>-0.12116211</x:v>
@@ -2603,25 +2603,25 @@
         <x:v>8.25</x:v>
       </x:c>
       <x:c r="C34" s="4" t="n">
-        <x:v>0.0703958</x:v>
+        <x:v>0.044878270000000005</x:v>
       </x:c>
       <x:c r="D34" s="4" t="n">
         <x:v>-0.08753875000000001</x:v>
       </x:c>
       <x:c r="E34" s="4" t="n">
-        <x:v>-0.00609143</x:v>
+        <x:v>-0.0137131</x:v>
       </x:c>
       <x:c r="F34" s="4" t="n">
         <x:v>-0.14165192</x:v>
       </x:c>
       <x:c r="G34" s="4" t="n">
-        <x:v>0.70355215</x:v>
+        <x:v>0.16451618</x:v>
       </x:c>
       <x:c r="H34" s="4" t="n">
         <x:v>0.05706486</x:v>
       </x:c>
       <x:c r="I34" s="4" t="n">
-        <x:v>0.01298729</x:v>
+        <x:v>-0.0067766300000000005</x:v>
       </x:c>
       <x:c r="J34" s="4" t="n">
         <x:v>-0.11531568</x:v>
@@ -2659,25 +2659,25 @@
         <x:v>8.5</x:v>
       </x:c>
       <x:c r="C35" s="4" t="n">
-        <x:v>0.06997463</x:v>
+        <x:v>0.04458181</x:v>
       </x:c>
       <x:c r="D35" s="4" t="n">
         <x:v>-0.08779089000000001</x:v>
       </x:c>
       <x:c r="E35" s="4" t="n">
-        <x:v>-0.00595619</x:v>
+        <x:v>-0.01362201</x:v>
       </x:c>
       <x:c r="F35" s="4" t="n">
         <x:v>-0.14188335</x:v>
       </x:c>
       <x:c r="G35" s="4" t="n">
-        <x:v>0.70160807</x:v>
+        <x:v>0.16036407</x:v>
       </x:c>
       <x:c r="H35" s="4" t="n">
         <x:v>0.05149625</x:v>
       </x:c>
       <x:c r="I35" s="4" t="n">
-        <x:v>0.01430439</x:v>
+        <x:v>-0.00553342</x:v>
       </x:c>
       <x:c r="J35" s="4" t="n">
         <x:v>-0.11499204</x:v>
@@ -2715,25 +2715,25 @@
         <x:v>8.75</x:v>
       </x:c>
       <x:c r="C36" s="4" t="n">
-        <x:v>0.07006228</x:v>
+        <x:v>0.04500741</x:v>
       </x:c>
       <x:c r="D36" s="4" t="n">
         <x:v>-0.08771841</x:v>
       </x:c>
       <x:c r="E36" s="4" t="n">
-        <x:v>-0.006062809999999999</x:v>
+        <x:v>-0.01394491</x:v>
       </x:c>
       <x:c r="F36" s="4" t="n">
         <x:v>-0.1425958</x:v>
       </x:c>
       <x:c r="G36" s="4" t="n">
-        <x:v>0.69839586</x:v>
+        <x:v>0.15462504</x:v>
       </x:c>
       <x:c r="H36" s="4" t="n">
         <x:v>0.04532014</x:v>
       </x:c>
       <x:c r="I36" s="4" t="n">
-        <x:v>0.01505572</x:v>
+        <x:v>-0.0051633600000000005</x:v>
       </x:c>
       <x:c r="J36" s="4" t="n">
         <x:v>-0.11513861</x:v>
@@ -2771,25 +2771,25 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="4" t="n">
-        <x:v>0.07019122</x:v>
+        <x:v>0.04549443</x:v>
       </x:c>
       <x:c r="D37" s="4" t="n">
         <x:v>-0.08754873999999999</x:v>
       </x:c>
       <x:c r="E37" s="4" t="n">
-        <x:v>-0.00597631</x:v>
+        <x:v>-0.013980999999999999</x:v>
       </x:c>
       <x:c r="F37" s="4" t="n">
         <x:v>-0.14325912000000002</x:v>
       </x:c>
       <x:c r="G37" s="4" t="n">
-        <x:v>0.69716669</x:v>
+        <x:v>0.15185879</x:v>
       </x:c>
       <x:c r="H37" s="4" t="n">
         <x:v>0.04225671</x:v>
       </x:c>
       <x:c r="I37" s="4" t="n">
-        <x:v>0.02279277</x:v>
+        <x:v>0.00406439</x:v>
       </x:c>
       <x:c r="J37" s="4" t="n">
         <x:v>-0.10706028999999999</x:v>
@@ -2827,25 +2827,25 @@
         <x:v>9.25</x:v>
       </x:c>
       <x:c r="C38" s="4" t="n">
-        <x:v>0.06995066</x:v>
+        <x:v>0.045434970000000005</x:v>
       </x:c>
       <x:c r="D38" s="4" t="n">
         <x:v>-0.08764687</x:v>
       </x:c>
       <x:c r="E38" s="4" t="n">
-        <x:v>-0.00553964</x:v>
+        <x:v>-0.01348161</x:v>
       </x:c>
       <x:c r="F38" s="4" t="n">
         <x:v>-0.14300353</x:v>
       </x:c>
       <x:c r="G38" s="4" t="n">
-        <x:v>0.69509513</x:v>
+        <x:v>0.14795714000000001</x:v>
       </x:c>
       <x:c r="H38" s="4" t="n">
         <x:v>0.03792561</x:v>
       </x:c>
       <x:c r="I38" s="4" t="n">
-        <x:v>0.017388840000000003</x:v>
+        <x:v>-0.00267833</x:v>
       </x:c>
       <x:c r="J38" s="4" t="n">
         <x:v>-0.11350634</x:v>
@@ -2883,25 +2883,25 @@
         <x:v>9.5</x:v>
       </x:c>
       <x:c r="C39" s="4" t="n">
-        <x:v>0.06995791999999999</x:v>
+        <x:v>0.04574687</x:v>
       </x:c>
       <x:c r="D39" s="4" t="n">
         <x:v>-0.08725006</x:v>
       </x:c>
       <x:c r="E39" s="4" t="n">
-        <x:v>-0.0044663</x:v>
+        <x:v>-0.01206821</x:v>
       </x:c>
       <x:c r="F39" s="4" t="n">
         <x:v>-0.14225091</x:v>
       </x:c>
       <x:c r="G39" s="4" t="n">
-        <x:v>0.6947220900000001</x:v>
+        <x:v>0.14639452</x:v>
       </x:c>
       <x:c r="H39" s="4" t="n">
         <x:v>0.0357702</x:v>
       </x:c>
       <x:c r="I39" s="4" t="n">
-        <x:v>0.01737249</x:v>
+        <x:v>-0.00307268</x:v>
       </x:c>
       <x:c r="J39" s="4" t="n">
         <x:v>-0.11531788000000001</x:v>
@@ -2939,25 +2939,25 @@
         <x:v>9.75</x:v>
       </x:c>
       <x:c r="C40" s="4" t="n">
-        <x:v>0.06985364</x:v>
+        <x:v>0.04586551</x:v>
       </x:c>
       <x:c r="D40" s="4" t="n">
         <x:v>-0.08703288</x:v>
       </x:c>
       <x:c r="E40" s="4" t="n">
-        <x:v>-0.005000360000000001</x:v>
+        <x:v>-0.0129453</x:v>
       </x:c>
       <x:c r="F40" s="4" t="n">
         <x:v>-0.14332185</x:v>
       </x:c>
       <x:c r="G40" s="4" t="n">
-        <x:v>0.69425637</x:v>
+        <x:v>0.14473527</x:v>
       </x:c>
       <x:c r="H40" s="4" t="n">
         <x:v>0.034069630000000004</x:v>
       </x:c>
       <x:c r="I40" s="4" t="n">
-        <x:v>0.018463419999999998</x:v>
+        <x:v>-0.0022140199999999997</x:v>
       </x:c>
       <x:c r="J40" s="4" t="n">
         <x:v>-0.11525044</x:v>
@@ -2995,25 +2995,25 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C41" s="4" t="n">
-        <x:v>0.06988264</x:v>
+        <x:v>0.04615957</x:v>
       </x:c>
       <x:c r="D41" s="4" t="n">
         <x:v>-0.08705237</x:v>
       </x:c>
       <x:c r="E41" s="4" t="n">
-        <x:v>-0.00515605</x:v>
+        <x:v>-0.01325015</x:v>
       </x:c>
       <x:c r="F41" s="4" t="n">
         <x:v>-0.14394679</x:v>
       </x:c>
       <x:c r="G41" s="4" t="n">
-        <x:v>0.6941789</x:v>
+        <x:v>0.1437518</x:v>
       </x:c>
       <x:c r="H41" s="4" t="n">
         <x:v>0.03233765</x:v>
       </x:c>
       <x:c r="I41" s="4" t="n">
-        <x:v>0.02430999</x:v>
+        <x:v>0.00519944</x:v>
       </x:c>
       <x:c r="J41" s="4" t="n">
         <x:v>-0.10899497999999999</x:v>
@@ -3045,9 +3045,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e82c5ea3946467b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d0d43b70f554158"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11a3fda857774ded"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d53d35483024bf5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>